<commit_message>
Automatická cesta u všech testovacích témat (16 prošlých verzí, 3 témata zastavená), podklad k hodnocení 40 verzí
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hodnoceni/hodnoceni-clanku.xlsx
+++ b/hodnoceni/hodnoceni-clanku.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Návod" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Hodnocení'!$A$6:$N$46</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Hodnocení'!$A$6:$N$56</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N46"/>
+  <dimension ref="A1:N56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1287,27 +1287,27 @@
     <row r="22">
       <c r="A22" s="10" t="inlineStr">
         <is>
-          <t>T3-A</t>
+          <t>T2-auto-A</t>
         </is>
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="C22" s="10" t="inlineStr">
         <is>
-          <t>Přestavba strahovských kolejí ČVUT</t>
+          <t>Nový kampus UK v Hradci Králové</t>
         </is>
       </c>
       <c r="D22" s="10" t="inlineStr">
         <is>
-          <t>Rozšířená rešerše</t>
+          <t>Automatická cesta</t>
         </is>
       </c>
       <c r="E22" s="10" t="inlineStr">
         <is>
-          <t>prošla po jedné opravě</t>
+          <t>prošla napoprvé</t>
         </is>
       </c>
       <c r="F22" s="10" t="inlineStr">
@@ -1330,22 +1330,22 @@
     <row r="23">
       <c r="A23" s="8" t="inlineStr">
         <is>
-          <t>T3-B</t>
+          <t>T2-auto-B</t>
         </is>
       </c>
       <c r="B23" s="8" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="C23" s="8" t="inlineStr">
         <is>
-          <t>Přestavba strahovských kolejí ČVUT</t>
+          <t>Nový kampus UK v Hradci Králové</t>
         </is>
       </c>
       <c r="D23" s="8" t="inlineStr">
         <is>
-          <t>Rozšířená rešerše</t>
+          <t>Automatická cesta</t>
         </is>
       </c>
       <c r="E23" s="8" t="inlineStr">
@@ -1373,27 +1373,27 @@
     <row r="24">
       <c r="A24" s="8" t="inlineStr">
         <is>
-          <t>T3-C</t>
+          <t>T2-auto-C</t>
         </is>
       </c>
       <c r="B24" s="8" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="C24" s="8" t="inlineStr">
         <is>
-          <t>Přestavba strahovských kolejí ČVUT</t>
+          <t>Nový kampus UK v Hradci Králové</t>
         </is>
       </c>
       <c r="D24" s="8" t="inlineStr">
         <is>
-          <t>Rozšířená rešerše</t>
+          <t>Automatická cesta</t>
         </is>
       </c>
       <c r="E24" s="8" t="inlineStr">
         <is>
-          <t>prošla po jedné opravě</t>
+          <t>prošla napoprvé</t>
         </is>
       </c>
       <c r="F24" s="8" t="inlineStr">
@@ -1416,22 +1416,22 @@
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>T3-D</t>
+          <t>T2-auto-D</t>
         </is>
       </c>
       <c r="B25" s="6" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="C25" s="6" t="inlineStr">
         <is>
-          <t>Přestavba strahovských kolejí ČVUT</t>
+          <t>Nový kampus UK v Hradci Králové</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>Rozšířená rešerše</t>
+          <t>Automatická cesta</t>
         </is>
       </c>
       <c r="E25" s="6" t="inlineStr">
@@ -1459,27 +1459,27 @@
     <row r="26">
       <c r="A26" s="8" t="inlineStr">
         <is>
-          <t>T3-E</t>
+          <t>T2-auto-E</t>
         </is>
       </c>
       <c r="B26" s="8" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="C26" s="8" t="inlineStr">
         <is>
-          <t>Přestavba strahovských kolejí ČVUT</t>
+          <t>Nový kampus UK v Hradci Králové</t>
         </is>
       </c>
       <c r="D26" s="8" t="inlineStr">
         <is>
-          <t>Rozšířená rešerše</t>
+          <t>Automatická cesta</t>
         </is>
       </c>
       <c r="E26" s="8" t="inlineStr">
         <is>
-          <t>prošla napoprvé</t>
+          <t>prošla po jedné opravě</t>
         </is>
       </c>
       <c r="F26" s="8" t="inlineStr">
@@ -1500,191 +1500,191 @@
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="12" t="inlineStr">
-        <is>
-          <t>T14-A</t>
-        </is>
-      </c>
-      <c r="B27" s="12" t="inlineStr">
-        <is>
-          <t>T14</t>
-        </is>
-      </c>
-      <c r="C27" s="12" t="inlineStr">
-        <is>
-          <t>Scio chce založit vlastní vysokou školu</t>
-        </is>
-      </c>
-      <c r="D27" s="12" t="inlineStr">
-        <is>
-          <t>Rozšířená rešerše</t>
-        </is>
-      </c>
-      <c r="E27" s="12" t="inlineStr">
+      <c r="A27" s="10" t="inlineStr">
+        <is>
+          <t>T3-A</t>
+        </is>
+      </c>
+      <c r="B27" s="10" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="C27" s="10" t="inlineStr">
+        <is>
+          <t>Přestavba strahovských kolejí ČVUT</t>
+        </is>
+      </c>
+      <c r="D27" s="10" t="inlineStr">
+        <is>
+          <t>Rozšířená rešerše</t>
+        </is>
+      </c>
+      <c r="E27" s="10" t="inlineStr">
+        <is>
+          <t>prošla po jedné opravě</t>
+        </is>
+      </c>
+      <c r="F27" s="10" t="inlineStr">
+        <is>
+          <t>ano</t>
+        </is>
+      </c>
+      <c r="G27" s="10" t="n"/>
+      <c r="H27" s="10" t="n"/>
+      <c r="I27" s="10" t="n"/>
+      <c r="J27" s="10" t="n"/>
+      <c r="K27" s="10" t="n"/>
+      <c r="L27" s="10" t="n"/>
+      <c r="M27" s="10" t="n"/>
+      <c r="N27" s="11">
+        <f>IF(COUNTA(G27:L27)&lt;&gt;COUNTIF(G27:L27,1)+COUNTIF(G27:L27,2)+COUNTIF(G27:L27,3)+COUNTIF(G27:L27,4)+COUNTIF(G27:L27,5),"jen celá čísla 1–5",IF(AND(COUNTA(H27:L27)&gt;0,COUNTA(G27)=0),"doplňte Celkově",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="8" t="inlineStr">
+        <is>
+          <t>T3-B</t>
+        </is>
+      </c>
+      <c r="B28" s="8" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>Přestavba strahovských kolejí ČVUT</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>Rozšířená rešerše</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>prošla po jedné opravě</t>
+        </is>
+      </c>
+      <c r="F28" s="8" t="inlineStr">
+        <is>
+          <t>ano</t>
+        </is>
+      </c>
+      <c r="G28" s="8" t="n"/>
+      <c r="H28" s="8" t="n"/>
+      <c r="I28" s="8" t="n"/>
+      <c r="J28" s="8" t="n"/>
+      <c r="K28" s="8" t="n"/>
+      <c r="L28" s="8" t="n"/>
+      <c r="M28" s="8" t="n"/>
+      <c r="N28" s="9">
+        <f>IF(COUNTA(G28:L28)&lt;&gt;COUNTIF(G28:L28,1)+COUNTIF(G28:L28,2)+COUNTIF(G28:L28,3)+COUNTIF(G28:L28,4)+COUNTIF(G28:L28,5),"jen celá čísla 1–5",IF(AND(COUNTA(H28:L28)&gt;0,COUNTA(G28)=0),"doplňte Celkově",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="8" t="inlineStr">
+        <is>
+          <t>T3-C</t>
+        </is>
+      </c>
+      <c r="B29" s="8" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="C29" s="8" t="inlineStr">
+        <is>
+          <t>Přestavba strahovských kolejí ČVUT</t>
+        </is>
+      </c>
+      <c r="D29" s="8" t="inlineStr">
+        <is>
+          <t>Rozšířená rešerše</t>
+        </is>
+      </c>
+      <c r="E29" s="8" t="inlineStr">
+        <is>
+          <t>prošla po jedné opravě</t>
+        </is>
+      </c>
+      <c r="F29" s="8" t="inlineStr">
+        <is>
+          <t>ano</t>
+        </is>
+      </c>
+      <c r="G29" s="8" t="n"/>
+      <c r="H29" s="8" t="n"/>
+      <c r="I29" s="8" t="n"/>
+      <c r="J29" s="8" t="n"/>
+      <c r="K29" s="8" t="n"/>
+      <c r="L29" s="8" t="n"/>
+      <c r="M29" s="8" t="n"/>
+      <c r="N29" s="9">
+        <f>IF(COUNTA(G29:L29)&lt;&gt;COUNTIF(G29:L29,1)+COUNTIF(G29:L29,2)+COUNTIF(G29:L29,3)+COUNTIF(G29:L29,4)+COUNTIF(G29:L29,5),"jen celá čísla 1–5",IF(AND(COUNTA(H29:L29)&gt;0,COUNTA(G29)=0),"doplňte Celkově",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="inlineStr">
+        <is>
+          <t>T3-D</t>
+        </is>
+      </c>
+      <c r="B30" s="6" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>Přestavba strahovských kolejí ČVUT</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="inlineStr">
+        <is>
+          <t>Rozšířená rešerše</t>
+        </is>
+      </c>
+      <c r="E30" s="6" t="inlineStr">
         <is>
           <t>neprošla – nehodnotí se</t>
         </is>
       </c>
-      <c r="F27" s="12" t="inlineStr">
+      <c r="F30" s="6" t="inlineStr">
         <is>
           <t>ne</t>
         </is>
       </c>
-      <c r="G27" s="12" t="n"/>
-      <c r="H27" s="12" t="n"/>
-      <c r="I27" s="12" t="n"/>
-      <c r="J27" s="12" t="n"/>
-      <c r="K27" s="12" t="n"/>
-      <c r="L27" s="12" t="n"/>
-      <c r="M27" s="12" t="n"/>
-      <c r="N27" s="13">
-        <f>IF(COUNTA(G27:L27)&gt;0,"neprošlá verze se nehodnotí","")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="6" t="inlineStr">
-        <is>
-          <t>T14-B</t>
-        </is>
-      </c>
-      <c r="B28" s="6" t="inlineStr">
-        <is>
-          <t>T14</t>
-        </is>
-      </c>
-      <c r="C28" s="6" t="inlineStr">
-        <is>
-          <t>Scio chce založit vlastní vysokou školu</t>
-        </is>
-      </c>
-      <c r="D28" s="6" t="inlineStr">
-        <is>
-          <t>Rozšířená rešerše</t>
-        </is>
-      </c>
-      <c r="E28" s="6" t="inlineStr">
-        <is>
-          <t>neprošla – nehodnotí se</t>
-        </is>
-      </c>
-      <c r="F28" s="6" t="inlineStr">
-        <is>
-          <t>ne</t>
-        </is>
-      </c>
-      <c r="G28" s="6" t="n"/>
-      <c r="H28" s="6" t="n"/>
-      <c r="I28" s="6" t="n"/>
-      <c r="J28" s="6" t="n"/>
-      <c r="K28" s="6" t="n"/>
-      <c r="L28" s="6" t="n"/>
-      <c r="M28" s="6" t="n"/>
-      <c r="N28" s="7">
-        <f>IF(COUNTA(G28:L28)&gt;0,"neprošlá verze se nehodnotí","")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="6" t="inlineStr">
-        <is>
-          <t>T14-C</t>
-        </is>
-      </c>
-      <c r="B29" s="6" t="inlineStr">
-        <is>
-          <t>T14</t>
-        </is>
-      </c>
-      <c r="C29" s="6" t="inlineStr">
-        <is>
-          <t>Scio chce založit vlastní vysokou školu</t>
-        </is>
-      </c>
-      <c r="D29" s="6" t="inlineStr">
-        <is>
-          <t>Rozšířená rešerše</t>
-        </is>
-      </c>
-      <c r="E29" s="6" t="inlineStr">
-        <is>
-          <t>neprošla – nehodnotí se</t>
-        </is>
-      </c>
-      <c r="F29" s="6" t="inlineStr">
-        <is>
-          <t>ne</t>
-        </is>
-      </c>
-      <c r="G29" s="6" t="n"/>
-      <c r="H29" s="6" t="n"/>
-      <c r="I29" s="6" t="n"/>
-      <c r="J29" s="6" t="n"/>
-      <c r="K29" s="6" t="n"/>
-      <c r="L29" s="6" t="n"/>
-      <c r="M29" s="6" t="n"/>
-      <c r="N29" s="7">
-        <f>IF(COUNTA(G29:L29)&gt;0,"neprošlá verze se nehodnotí","")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="8" t="inlineStr">
-        <is>
-          <t>T14-D</t>
-        </is>
-      </c>
-      <c r="B30" s="8" t="inlineStr">
-        <is>
-          <t>T14</t>
-        </is>
-      </c>
-      <c r="C30" s="8" t="inlineStr">
-        <is>
-          <t>Scio chce založit vlastní vysokou školu</t>
-        </is>
-      </c>
-      <c r="D30" s="8" t="inlineStr">
-        <is>
-          <t>Rozšířená rešerše</t>
-        </is>
-      </c>
-      <c r="E30" s="8" t="inlineStr">
-        <is>
-          <t>prošla po jedné opravě</t>
-        </is>
-      </c>
-      <c r="F30" s="8" t="inlineStr">
-        <is>
-          <t>ano</t>
-        </is>
-      </c>
-      <c r="G30" s="8" t="n"/>
-      <c r="H30" s="8" t="n"/>
-      <c r="I30" s="8" t="n"/>
-      <c r="J30" s="8" t="n"/>
-      <c r="K30" s="8" t="n"/>
-      <c r="L30" s="8" t="n"/>
-      <c r="M30" s="8" t="n"/>
-      <c r="N30" s="9">
-        <f>IF(COUNTA(G30:L30)&lt;&gt;COUNTIF(G30:L30,1)+COUNTIF(G30:L30,2)+COUNTIF(G30:L30,3)+COUNTIF(G30:L30,4)+COUNTIF(G30:L30,5),"jen celá čísla 1–5",IF(AND(COUNTA(H30:L30)&gt;0,COUNTA(G30)=0),"doplňte Celkově",""))</f>
+      <c r="G30" s="6" t="n"/>
+      <c r="H30" s="6" t="n"/>
+      <c r="I30" s="6" t="n"/>
+      <c r="J30" s="6" t="n"/>
+      <c r="K30" s="6" t="n"/>
+      <c r="L30" s="6" t="n"/>
+      <c r="M30" s="6" t="n"/>
+      <c r="N30" s="7">
+        <f>IF(COUNTA(G30:L30)&gt;0,"neprošlá verze se nehodnotí","")</f>
         <v/>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="8" t="inlineStr">
         <is>
-          <t>T14-E</t>
+          <t>T3-E</t>
         </is>
       </c>
       <c r="B31" s="8" t="inlineStr">
         <is>
-          <t>T14</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="C31" s="8" t="inlineStr">
         <is>
-          <t>Scio chce založit vlastní vysokou školu</t>
+          <t>Přestavba strahovských kolejí ČVUT</t>
         </is>
       </c>
       <c r="D31" s="8" t="inlineStr">
@@ -1694,7 +1694,7 @@
       </c>
       <c r="E31" s="8" t="inlineStr">
         <is>
-          <t>prošla po jedné opravě</t>
+          <t>prošla napoprvé</t>
         </is>
       </c>
       <c r="F31" s="8" t="inlineStr">
@@ -1715,62 +1715,62 @@
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="12" t="inlineStr">
-        <is>
-          <t>T15-auto-A</t>
-        </is>
-      </c>
-      <c r="B32" s="12" t="inlineStr">
-        <is>
-          <t>T15</t>
-        </is>
-      </c>
-      <c r="C32" s="12" t="inlineStr">
-        <is>
-          <t>Univerzitní hokejová derby</t>
-        </is>
-      </c>
-      <c r="D32" s="12" t="inlineStr">
+      <c r="A32" s="10" t="inlineStr">
+        <is>
+          <t>T3-auto-A</t>
+        </is>
+      </c>
+      <c r="B32" s="10" t="inlineStr">
+        <is>
+          <t>T3</t>
+        </is>
+      </c>
+      <c r="C32" s="10" t="inlineStr">
+        <is>
+          <t>Přestavba strahovských kolejí ČVUT</t>
+        </is>
+      </c>
+      <c r="D32" s="10" t="inlineStr">
         <is>
           <t>Automatická cesta</t>
         </is>
       </c>
-      <c r="E32" s="12" t="inlineStr">
-        <is>
-          <t>neprošla – nehodnotí se</t>
-        </is>
-      </c>
-      <c r="F32" s="12" t="inlineStr">
-        <is>
-          <t>ne</t>
-        </is>
-      </c>
-      <c r="G32" s="12" t="n"/>
-      <c r="H32" s="12" t="n"/>
-      <c r="I32" s="12" t="n"/>
-      <c r="J32" s="12" t="n"/>
-      <c r="K32" s="12" t="n"/>
-      <c r="L32" s="12" t="n"/>
-      <c r="M32" s="12" t="n"/>
-      <c r="N32" s="13">
-        <f>IF(COUNTA(G32:L32)&gt;0,"neprošlá verze se nehodnotí","")</f>
+      <c r="E32" s="10" t="inlineStr">
+        <is>
+          <t>prošla po jedné opravě</t>
+        </is>
+      </c>
+      <c r="F32" s="10" t="inlineStr">
+        <is>
+          <t>ano</t>
+        </is>
+      </c>
+      <c r="G32" s="10" t="n"/>
+      <c r="H32" s="10" t="n"/>
+      <c r="I32" s="10" t="n"/>
+      <c r="J32" s="10" t="n"/>
+      <c r="K32" s="10" t="n"/>
+      <c r="L32" s="10" t="n"/>
+      <c r="M32" s="10" t="n"/>
+      <c r="N32" s="11">
+        <f>IF(COUNTA(G32:L32)&lt;&gt;COUNTIF(G32:L32,1)+COUNTIF(G32:L32,2)+COUNTIF(G32:L32,3)+COUNTIF(G32:L32,4)+COUNTIF(G32:L32,5),"jen celá čísla 1–5",IF(AND(COUNTA(H32:L32)&gt;0,COUNTA(G32)=0),"doplňte Celkově",""))</f>
         <v/>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="8" t="inlineStr">
         <is>
-          <t>T15-auto-B</t>
+          <t>T3-auto-B</t>
         </is>
       </c>
       <c r="B33" s="8" t="inlineStr">
         <is>
-          <t>T15</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="C33" s="8" t="inlineStr">
         <is>
-          <t>Univerzitní hokejová derby</t>
+          <t>Přestavba strahovských kolejí ČVUT</t>
         </is>
       </c>
       <c r="D33" s="8" t="inlineStr">
@@ -1803,17 +1803,17 @@
     <row r="34">
       <c r="A34" s="8" t="inlineStr">
         <is>
-          <t>T15-auto-C</t>
+          <t>T3-auto-C</t>
         </is>
       </c>
       <c r="B34" s="8" t="inlineStr">
         <is>
-          <t>T15</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="C34" s="8" t="inlineStr">
         <is>
-          <t>Univerzitní hokejová derby</t>
+          <t>Přestavba strahovských kolejí ČVUT</t>
         </is>
       </c>
       <c r="D34" s="8" t="inlineStr">
@@ -1823,7 +1823,7 @@
       </c>
       <c r="E34" s="8" t="inlineStr">
         <is>
-          <t>prošla napoprvé</t>
+          <t>prošla po jedné opravě</t>
         </is>
       </c>
       <c r="F34" s="8" t="inlineStr">
@@ -1846,17 +1846,17 @@
     <row r="35">
       <c r="A35" s="8" t="inlineStr">
         <is>
-          <t>T15-auto-D</t>
+          <t>T3-auto-D</t>
         </is>
       </c>
       <c r="B35" s="8" t="inlineStr">
         <is>
-          <t>T15</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="C35" s="8" t="inlineStr">
         <is>
-          <t>Univerzitní hokejová derby</t>
+          <t>Přestavba strahovských kolejí ČVUT</t>
         </is>
       </c>
       <c r="D35" s="8" t="inlineStr">
@@ -1866,7 +1866,7 @@
       </c>
       <c r="E35" s="8" t="inlineStr">
         <is>
-          <t>prošla napoprvé</t>
+          <t>prošla po jedné opravě</t>
         </is>
       </c>
       <c r="F35" s="8" t="inlineStr">
@@ -1889,17 +1889,17 @@
     <row r="36">
       <c r="A36" s="8" t="inlineStr">
         <is>
-          <t>T15-auto-E</t>
+          <t>T3-auto-E</t>
         </is>
       </c>
       <c r="B36" s="8" t="inlineStr">
         <is>
-          <t>T15</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="C36" s="8" t="inlineStr">
         <is>
-          <t>Univerzitní hokejová derby</t>
+          <t>Přestavba strahovských kolejí ČVUT</t>
         </is>
       </c>
       <c r="D36" s="8" t="inlineStr">
@@ -1930,148 +1930,148 @@
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="10" t="inlineStr">
-        <is>
-          <t>T16-A</t>
-        </is>
-      </c>
-      <c r="B37" s="10" t="inlineStr">
-        <is>
-          <t>T16</t>
-        </is>
-      </c>
-      <c r="C37" s="10" t="inlineStr">
-        <is>
-          <t>Neúspěch u maturity: jak na další pokus</t>
-        </is>
-      </c>
-      <c r="D37" s="10" t="inlineStr">
-        <is>
-          <t>Rozšířená rešerše</t>
-        </is>
-      </c>
-      <c r="E37" s="10" t="inlineStr">
-        <is>
-          <t>prošla napoprvé</t>
-        </is>
-      </c>
-      <c r="F37" s="10" t="inlineStr">
-        <is>
-          <t>ano</t>
-        </is>
-      </c>
-      <c r="G37" s="10" t="n"/>
-      <c r="H37" s="10" t="n"/>
-      <c r="I37" s="10" t="n"/>
-      <c r="J37" s="10" t="n"/>
-      <c r="K37" s="10" t="n"/>
-      <c r="L37" s="10" t="n"/>
-      <c r="M37" s="10" t="n"/>
-      <c r="N37" s="11">
-        <f>IF(COUNTA(G37:L37)&lt;&gt;COUNTIF(G37:L37,1)+COUNTIF(G37:L37,2)+COUNTIF(G37:L37,3)+COUNTIF(G37:L37,4)+COUNTIF(G37:L37,5),"jen celá čísla 1–5",IF(AND(COUNTA(H37:L37)&gt;0,COUNTA(G37)=0),"doplňte Celkově",""))</f>
+      <c r="A37" s="12" t="inlineStr">
+        <is>
+          <t>T14-A</t>
+        </is>
+      </c>
+      <c r="B37" s="12" t="inlineStr">
+        <is>
+          <t>T14</t>
+        </is>
+      </c>
+      <c r="C37" s="12" t="inlineStr">
+        <is>
+          <t>Scio chce založit vlastní vysokou školu</t>
+        </is>
+      </c>
+      <c r="D37" s="12" t="inlineStr">
+        <is>
+          <t>Rozšířená rešerše</t>
+        </is>
+      </c>
+      <c r="E37" s="12" t="inlineStr">
+        <is>
+          <t>neprošla – nehodnotí se</t>
+        </is>
+      </c>
+      <c r="F37" s="12" t="inlineStr">
+        <is>
+          <t>ne</t>
+        </is>
+      </c>
+      <c r="G37" s="12" t="n"/>
+      <c r="H37" s="12" t="n"/>
+      <c r="I37" s="12" t="n"/>
+      <c r="J37" s="12" t="n"/>
+      <c r="K37" s="12" t="n"/>
+      <c r="L37" s="12" t="n"/>
+      <c r="M37" s="12" t="n"/>
+      <c r="N37" s="13">
+        <f>IF(COUNTA(G37:L37)&gt;0,"neprošlá verze se nehodnotí","")</f>
         <v/>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="8" t="inlineStr">
-        <is>
-          <t>T16-B</t>
-        </is>
-      </c>
-      <c r="B38" s="8" t="inlineStr">
-        <is>
-          <t>T16</t>
-        </is>
-      </c>
-      <c r="C38" s="8" t="inlineStr">
-        <is>
-          <t>Neúspěch u maturity: jak na další pokus</t>
-        </is>
-      </c>
-      <c r="D38" s="8" t="inlineStr">
-        <is>
-          <t>Rozšířená rešerše</t>
-        </is>
-      </c>
-      <c r="E38" s="8" t="inlineStr">
-        <is>
-          <t>prošla po jedné opravě</t>
-        </is>
-      </c>
-      <c r="F38" s="8" t="inlineStr">
-        <is>
-          <t>ano</t>
-        </is>
-      </c>
-      <c r="G38" s="8" t="n"/>
-      <c r="H38" s="8" t="n"/>
-      <c r="I38" s="8" t="n"/>
-      <c r="J38" s="8" t="n"/>
-      <c r="K38" s="8" t="n"/>
-      <c r="L38" s="8" t="n"/>
-      <c r="M38" s="8" t="n"/>
-      <c r="N38" s="9">
-        <f>IF(COUNTA(G38:L38)&lt;&gt;COUNTIF(G38:L38,1)+COUNTIF(G38:L38,2)+COUNTIF(G38:L38,3)+COUNTIF(G38:L38,4)+COUNTIF(G38:L38,5),"jen celá čísla 1–5",IF(AND(COUNTA(H38:L38)&gt;0,COUNTA(G38)=0),"doplňte Celkově",""))</f>
+      <c r="A38" s="6" t="inlineStr">
+        <is>
+          <t>T14-B</t>
+        </is>
+      </c>
+      <c r="B38" s="6" t="inlineStr">
+        <is>
+          <t>T14</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>Scio chce založit vlastní vysokou školu</t>
+        </is>
+      </c>
+      <c r="D38" s="6" t="inlineStr">
+        <is>
+          <t>Rozšířená rešerše</t>
+        </is>
+      </c>
+      <c r="E38" s="6" t="inlineStr">
+        <is>
+          <t>neprošla – nehodnotí se</t>
+        </is>
+      </c>
+      <c r="F38" s="6" t="inlineStr">
+        <is>
+          <t>ne</t>
+        </is>
+      </c>
+      <c r="G38" s="6" t="n"/>
+      <c r="H38" s="6" t="n"/>
+      <c r="I38" s="6" t="n"/>
+      <c r="J38" s="6" t="n"/>
+      <c r="K38" s="6" t="n"/>
+      <c r="L38" s="6" t="n"/>
+      <c r="M38" s="6" t="n"/>
+      <c r="N38" s="7">
+        <f>IF(COUNTA(G38:L38)&gt;0,"neprošlá verze se nehodnotí","")</f>
         <v/>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="8" t="inlineStr">
-        <is>
-          <t>T16-C</t>
-        </is>
-      </c>
-      <c r="B39" s="8" t="inlineStr">
-        <is>
-          <t>T16</t>
-        </is>
-      </c>
-      <c r="C39" s="8" t="inlineStr">
-        <is>
-          <t>Neúspěch u maturity: jak na další pokus</t>
-        </is>
-      </c>
-      <c r="D39" s="8" t="inlineStr">
-        <is>
-          <t>Rozšířená rešerše</t>
-        </is>
-      </c>
-      <c r="E39" s="8" t="inlineStr">
-        <is>
-          <t>prošla po jedné opravě</t>
-        </is>
-      </c>
-      <c r="F39" s="8" t="inlineStr">
-        <is>
-          <t>ano</t>
-        </is>
-      </c>
-      <c r="G39" s="8" t="n"/>
-      <c r="H39" s="8" t="n"/>
-      <c r="I39" s="8" t="n"/>
-      <c r="J39" s="8" t="n"/>
-      <c r="K39" s="8" t="n"/>
-      <c r="L39" s="8" t="n"/>
-      <c r="M39" s="8" t="n"/>
-      <c r="N39" s="9">
-        <f>IF(COUNTA(G39:L39)&lt;&gt;COUNTIF(G39:L39,1)+COUNTIF(G39:L39,2)+COUNTIF(G39:L39,3)+COUNTIF(G39:L39,4)+COUNTIF(G39:L39,5),"jen celá čísla 1–5",IF(AND(COUNTA(H39:L39)&gt;0,COUNTA(G39)=0),"doplňte Celkově",""))</f>
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t>T14-C</t>
+        </is>
+      </c>
+      <c r="B39" s="6" t="inlineStr">
+        <is>
+          <t>T14</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>Scio chce založit vlastní vysokou školu</t>
+        </is>
+      </c>
+      <c r="D39" s="6" t="inlineStr">
+        <is>
+          <t>Rozšířená rešerše</t>
+        </is>
+      </c>
+      <c r="E39" s="6" t="inlineStr">
+        <is>
+          <t>neprošla – nehodnotí se</t>
+        </is>
+      </c>
+      <c r="F39" s="6" t="inlineStr">
+        <is>
+          <t>ne</t>
+        </is>
+      </c>
+      <c r="G39" s="6" t="n"/>
+      <c r="H39" s="6" t="n"/>
+      <c r="I39" s="6" t="n"/>
+      <c r="J39" s="6" t="n"/>
+      <c r="K39" s="6" t="n"/>
+      <c r="L39" s="6" t="n"/>
+      <c r="M39" s="6" t="n"/>
+      <c r="N39" s="7">
+        <f>IF(COUNTA(G39:L39)&gt;0,"neprošlá verze se nehodnotí","")</f>
         <v/>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="8" t="inlineStr">
         <is>
-          <t>T16-D</t>
+          <t>T14-D</t>
         </is>
       </c>
       <c r="B40" s="8" t="inlineStr">
         <is>
-          <t>T16</t>
+          <t>T14</t>
         </is>
       </c>
       <c r="C40" s="8" t="inlineStr">
         <is>
-          <t>Neúspěch u maturity: jak na další pokus</t>
+          <t>Scio chce založit vlastní vysokou školu</t>
         </is>
       </c>
       <c r="D40" s="8" t="inlineStr">
@@ -2104,17 +2104,17 @@
     <row r="41">
       <c r="A41" s="8" t="inlineStr">
         <is>
-          <t>T16-E</t>
+          <t>T14-E</t>
         </is>
       </c>
       <c r="B41" s="8" t="inlineStr">
         <is>
-          <t>T16</t>
+          <t>T14</t>
         </is>
       </c>
       <c r="C41" s="8" t="inlineStr">
         <is>
-          <t>Neúspěch u maturity: jak na další pokus</t>
+          <t>Scio chce založit vlastní vysokou školu</t>
         </is>
       </c>
       <c r="D41" s="8" t="inlineStr">
@@ -2124,7 +2124,7 @@
       </c>
       <c r="E41" s="8" t="inlineStr">
         <is>
-          <t>prošla napoprvé</t>
+          <t>prošla po jedné opravě</t>
         </is>
       </c>
       <c r="F41" s="8" t="inlineStr">
@@ -2145,67 +2145,67 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="10" t="inlineStr">
-        <is>
-          <t>T17-A</t>
-        </is>
-      </c>
-      <c r="B42" s="10" t="inlineStr">
-        <is>
-          <t>T17</t>
-        </is>
-      </c>
-      <c r="C42" s="10" t="inlineStr">
-        <is>
-          <t>Farmaceutická fakulta UK v novém kampusu v Hradci Králové: první týdny</t>
-        </is>
-      </c>
-      <c r="D42" s="10" t="inlineStr">
-        <is>
-          <t>Rozšířená rešerše</t>
-        </is>
-      </c>
-      <c r="E42" s="10" t="inlineStr">
-        <is>
-          <t>prošla napoprvé</t>
-        </is>
-      </c>
-      <c r="F42" s="10" t="inlineStr">
-        <is>
-          <t>ano</t>
-        </is>
-      </c>
-      <c r="G42" s="10" t="n"/>
-      <c r="H42" s="10" t="n"/>
-      <c r="I42" s="10" t="n"/>
-      <c r="J42" s="10" t="n"/>
-      <c r="K42" s="10" t="n"/>
-      <c r="L42" s="10" t="n"/>
-      <c r="M42" s="10" t="n"/>
-      <c r="N42" s="11">
-        <f>IF(COUNTA(G42:L42)&lt;&gt;COUNTIF(G42:L42,1)+COUNTIF(G42:L42,2)+COUNTIF(G42:L42,3)+COUNTIF(G42:L42,4)+COUNTIF(G42:L42,5),"jen celá čísla 1–5",IF(AND(COUNTA(H42:L42)&gt;0,COUNTA(G42)=0),"doplňte Celkově",""))</f>
+      <c r="A42" s="12" t="inlineStr">
+        <is>
+          <t>T15-auto-A</t>
+        </is>
+      </c>
+      <c r="B42" s="12" t="inlineStr">
+        <is>
+          <t>T15</t>
+        </is>
+      </c>
+      <c r="C42" s="12" t="inlineStr">
+        <is>
+          <t>Univerzitní hokejová derby</t>
+        </is>
+      </c>
+      <c r="D42" s="12" t="inlineStr">
+        <is>
+          <t>Automatická cesta</t>
+        </is>
+      </c>
+      <c r="E42" s="12" t="inlineStr">
+        <is>
+          <t>neprošla – nehodnotí se</t>
+        </is>
+      </c>
+      <c r="F42" s="12" t="inlineStr">
+        <is>
+          <t>ne</t>
+        </is>
+      </c>
+      <c r="G42" s="12" t="n"/>
+      <c r="H42" s="12" t="n"/>
+      <c r="I42" s="12" t="n"/>
+      <c r="J42" s="12" t="n"/>
+      <c r="K42" s="12" t="n"/>
+      <c r="L42" s="12" t="n"/>
+      <c r="M42" s="12" t="n"/>
+      <c r="N42" s="13">
+        <f>IF(COUNTA(G42:L42)&gt;0,"neprošlá verze se nehodnotí","")</f>
         <v/>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="8" t="inlineStr">
         <is>
-          <t>T17-B</t>
+          <t>T15-auto-B</t>
         </is>
       </c>
       <c r="B43" s="8" t="inlineStr">
         <is>
-          <t>T17</t>
+          <t>T15</t>
         </is>
       </c>
       <c r="C43" s="8" t="inlineStr">
         <is>
-          <t>Farmaceutická fakulta UK v novém kampusu v Hradci Králové: první týdny</t>
+          <t>Univerzitní hokejová derby</t>
         </is>
       </c>
       <c r="D43" s="8" t="inlineStr">
         <is>
-          <t>Rozšířená rešerše</t>
+          <t>Automatická cesta</t>
         </is>
       </c>
       <c r="E43" s="8" t="inlineStr">
@@ -2233,27 +2233,27 @@
     <row r="44">
       <c r="A44" s="8" t="inlineStr">
         <is>
-          <t>T17-C</t>
+          <t>T15-auto-C</t>
         </is>
       </c>
       <c r="B44" s="8" t="inlineStr">
         <is>
-          <t>T17</t>
+          <t>T15</t>
         </is>
       </c>
       <c r="C44" s="8" t="inlineStr">
         <is>
-          <t>Farmaceutická fakulta UK v novém kampusu v Hradci Králové: první týdny</t>
+          <t>Univerzitní hokejová derby</t>
         </is>
       </c>
       <c r="D44" s="8" t="inlineStr">
         <is>
-          <t>Rozšířená rešerše</t>
+          <t>Automatická cesta</t>
         </is>
       </c>
       <c r="E44" s="8" t="inlineStr">
         <is>
-          <t>prošla po jedné opravě</t>
+          <t>prošla napoprvé</t>
         </is>
       </c>
       <c r="F44" s="8" t="inlineStr">
@@ -2276,27 +2276,27 @@
     <row r="45">
       <c r="A45" s="8" t="inlineStr">
         <is>
-          <t>T17-D</t>
+          <t>T15-auto-D</t>
         </is>
       </c>
       <c r="B45" s="8" t="inlineStr">
         <is>
-          <t>T17</t>
+          <t>T15</t>
         </is>
       </c>
       <c r="C45" s="8" t="inlineStr">
         <is>
-          <t>Farmaceutická fakulta UK v novém kampusu v Hradci Králové: první týdny</t>
+          <t>Univerzitní hokejová derby</t>
         </is>
       </c>
       <c r="D45" s="8" t="inlineStr">
         <is>
-          <t>Rozšířená rešerše</t>
+          <t>Automatická cesta</t>
         </is>
       </c>
       <c r="E45" s="8" t="inlineStr">
         <is>
-          <t>prošla po jedné opravě</t>
+          <t>prošla napoprvé</t>
         </is>
       </c>
       <c r="F45" s="8" t="inlineStr">
@@ -2319,27 +2319,27 @@
     <row r="46">
       <c r="A46" s="8" t="inlineStr">
         <is>
-          <t>T17-E</t>
+          <t>T15-auto-E</t>
         </is>
       </c>
       <c r="B46" s="8" t="inlineStr">
         <is>
-          <t>T17</t>
+          <t>T15</t>
         </is>
       </c>
       <c r="C46" s="8" t="inlineStr">
         <is>
-          <t>Farmaceutická fakulta UK v novém kampusu v Hradci Králové: první týdny</t>
+          <t>Univerzitní hokejová derby</t>
         </is>
       </c>
       <c r="D46" s="8" t="inlineStr">
         <is>
-          <t>Rozšířená rešerše</t>
+          <t>Automatická cesta</t>
         </is>
       </c>
       <c r="E46" s="8" t="inlineStr">
         <is>
-          <t>prošla po jedné opravě</t>
+          <t>prošla napoprvé</t>
         </is>
       </c>
       <c r="F46" s="8" t="inlineStr">
@@ -2359,9 +2359,439 @@
         <v/>
       </c>
     </row>
+    <row r="47">
+      <c r="A47" s="10" t="inlineStr">
+        <is>
+          <t>T16-A</t>
+        </is>
+      </c>
+      <c r="B47" s="10" t="inlineStr">
+        <is>
+          <t>T16</t>
+        </is>
+      </c>
+      <c r="C47" s="10" t="inlineStr">
+        <is>
+          <t>Neúspěch u maturity: jak na další pokus</t>
+        </is>
+      </c>
+      <c r="D47" s="10" t="inlineStr">
+        <is>
+          <t>Rozšířená rešerše</t>
+        </is>
+      </c>
+      <c r="E47" s="10" t="inlineStr">
+        <is>
+          <t>prošla napoprvé</t>
+        </is>
+      </c>
+      <c r="F47" s="10" t="inlineStr">
+        <is>
+          <t>ano</t>
+        </is>
+      </c>
+      <c r="G47" s="10" t="n"/>
+      <c r="H47" s="10" t="n"/>
+      <c r="I47" s="10" t="n"/>
+      <c r="J47" s="10" t="n"/>
+      <c r="K47" s="10" t="n"/>
+      <c r="L47" s="10" t="n"/>
+      <c r="M47" s="10" t="n"/>
+      <c r="N47" s="11">
+        <f>IF(COUNTA(G47:L47)&lt;&gt;COUNTIF(G47:L47,1)+COUNTIF(G47:L47,2)+COUNTIF(G47:L47,3)+COUNTIF(G47:L47,4)+COUNTIF(G47:L47,5),"jen celá čísla 1–5",IF(AND(COUNTA(H47:L47)&gt;0,COUNTA(G47)=0),"doplňte Celkově",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="8" t="inlineStr">
+        <is>
+          <t>T16-B</t>
+        </is>
+      </c>
+      <c r="B48" s="8" t="inlineStr">
+        <is>
+          <t>T16</t>
+        </is>
+      </c>
+      <c r="C48" s="8" t="inlineStr">
+        <is>
+          <t>Neúspěch u maturity: jak na další pokus</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="inlineStr">
+        <is>
+          <t>Rozšířená rešerše</t>
+        </is>
+      </c>
+      <c r="E48" s="8" t="inlineStr">
+        <is>
+          <t>prošla po jedné opravě</t>
+        </is>
+      </c>
+      <c r="F48" s="8" t="inlineStr">
+        <is>
+          <t>ano</t>
+        </is>
+      </c>
+      <c r="G48" s="8" t="n"/>
+      <c r="H48" s="8" t="n"/>
+      <c r="I48" s="8" t="n"/>
+      <c r="J48" s="8" t="n"/>
+      <c r="K48" s="8" t="n"/>
+      <c r="L48" s="8" t="n"/>
+      <c r="M48" s="8" t="n"/>
+      <c r="N48" s="9">
+        <f>IF(COUNTA(G48:L48)&lt;&gt;COUNTIF(G48:L48,1)+COUNTIF(G48:L48,2)+COUNTIF(G48:L48,3)+COUNTIF(G48:L48,4)+COUNTIF(G48:L48,5),"jen celá čísla 1–5",IF(AND(COUNTA(H48:L48)&gt;0,COUNTA(G48)=0),"doplňte Celkově",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="8" t="inlineStr">
+        <is>
+          <t>T16-C</t>
+        </is>
+      </c>
+      <c r="B49" s="8" t="inlineStr">
+        <is>
+          <t>T16</t>
+        </is>
+      </c>
+      <c r="C49" s="8" t="inlineStr">
+        <is>
+          <t>Neúspěch u maturity: jak na další pokus</t>
+        </is>
+      </c>
+      <c r="D49" s="8" t="inlineStr">
+        <is>
+          <t>Rozšířená rešerše</t>
+        </is>
+      </c>
+      <c r="E49" s="8" t="inlineStr">
+        <is>
+          <t>prošla po jedné opravě</t>
+        </is>
+      </c>
+      <c r="F49" s="8" t="inlineStr">
+        <is>
+          <t>ano</t>
+        </is>
+      </c>
+      <c r="G49" s="8" t="n"/>
+      <c r="H49" s="8" t="n"/>
+      <c r="I49" s="8" t="n"/>
+      <c r="J49" s="8" t="n"/>
+      <c r="K49" s="8" t="n"/>
+      <c r="L49" s="8" t="n"/>
+      <c r="M49" s="8" t="n"/>
+      <c r="N49" s="9">
+        <f>IF(COUNTA(G49:L49)&lt;&gt;COUNTIF(G49:L49,1)+COUNTIF(G49:L49,2)+COUNTIF(G49:L49,3)+COUNTIF(G49:L49,4)+COUNTIF(G49:L49,5),"jen celá čísla 1–5",IF(AND(COUNTA(H49:L49)&gt;0,COUNTA(G49)=0),"doplňte Celkově",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="8" t="inlineStr">
+        <is>
+          <t>T16-D</t>
+        </is>
+      </c>
+      <c r="B50" s="8" t="inlineStr">
+        <is>
+          <t>T16</t>
+        </is>
+      </c>
+      <c r="C50" s="8" t="inlineStr">
+        <is>
+          <t>Neúspěch u maturity: jak na další pokus</t>
+        </is>
+      </c>
+      <c r="D50" s="8" t="inlineStr">
+        <is>
+          <t>Rozšířená rešerše</t>
+        </is>
+      </c>
+      <c r="E50" s="8" t="inlineStr">
+        <is>
+          <t>prošla po jedné opravě</t>
+        </is>
+      </c>
+      <c r="F50" s="8" t="inlineStr">
+        <is>
+          <t>ano</t>
+        </is>
+      </c>
+      <c r="G50" s="8" t="n"/>
+      <c r="H50" s="8" t="n"/>
+      <c r="I50" s="8" t="n"/>
+      <c r="J50" s="8" t="n"/>
+      <c r="K50" s="8" t="n"/>
+      <c r="L50" s="8" t="n"/>
+      <c r="M50" s="8" t="n"/>
+      <c r="N50" s="9">
+        <f>IF(COUNTA(G50:L50)&lt;&gt;COUNTIF(G50:L50,1)+COUNTIF(G50:L50,2)+COUNTIF(G50:L50,3)+COUNTIF(G50:L50,4)+COUNTIF(G50:L50,5),"jen celá čísla 1–5",IF(AND(COUNTA(H50:L50)&gt;0,COUNTA(G50)=0),"doplňte Celkově",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="8" t="inlineStr">
+        <is>
+          <t>T16-E</t>
+        </is>
+      </c>
+      <c r="B51" s="8" t="inlineStr">
+        <is>
+          <t>T16</t>
+        </is>
+      </c>
+      <c r="C51" s="8" t="inlineStr">
+        <is>
+          <t>Neúspěch u maturity: jak na další pokus</t>
+        </is>
+      </c>
+      <c r="D51" s="8" t="inlineStr">
+        <is>
+          <t>Rozšířená rešerše</t>
+        </is>
+      </c>
+      <c r="E51" s="8" t="inlineStr">
+        <is>
+          <t>prošla napoprvé</t>
+        </is>
+      </c>
+      <c r="F51" s="8" t="inlineStr">
+        <is>
+          <t>ano</t>
+        </is>
+      </c>
+      <c r="G51" s="8" t="n"/>
+      <c r="H51" s="8" t="n"/>
+      <c r="I51" s="8" t="n"/>
+      <c r="J51" s="8" t="n"/>
+      <c r="K51" s="8" t="n"/>
+      <c r="L51" s="8" t="n"/>
+      <c r="M51" s="8" t="n"/>
+      <c r="N51" s="9">
+        <f>IF(COUNTA(G51:L51)&lt;&gt;COUNTIF(G51:L51,1)+COUNTIF(G51:L51,2)+COUNTIF(G51:L51,3)+COUNTIF(G51:L51,4)+COUNTIF(G51:L51,5),"jen celá čísla 1–5",IF(AND(COUNTA(H51:L51)&gt;0,COUNTA(G51)=0),"doplňte Celkově",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="10" t="inlineStr">
+        <is>
+          <t>T17-A</t>
+        </is>
+      </c>
+      <c r="B52" s="10" t="inlineStr">
+        <is>
+          <t>T17</t>
+        </is>
+      </c>
+      <c r="C52" s="10" t="inlineStr">
+        <is>
+          <t>Farmaceutická fakulta UK v novém kampusu v Hradci Králové: první týdny</t>
+        </is>
+      </c>
+      <c r="D52" s="10" t="inlineStr">
+        <is>
+          <t>Rozšířená rešerše</t>
+        </is>
+      </c>
+      <c r="E52" s="10" t="inlineStr">
+        <is>
+          <t>prošla napoprvé</t>
+        </is>
+      </c>
+      <c r="F52" s="10" t="inlineStr">
+        <is>
+          <t>ano</t>
+        </is>
+      </c>
+      <c r="G52" s="10" t="n"/>
+      <c r="H52" s="10" t="n"/>
+      <c r="I52" s="10" t="n"/>
+      <c r="J52" s="10" t="n"/>
+      <c r="K52" s="10" t="n"/>
+      <c r="L52" s="10" t="n"/>
+      <c r="M52" s="10" t="n"/>
+      <c r="N52" s="11">
+        <f>IF(COUNTA(G52:L52)&lt;&gt;COUNTIF(G52:L52,1)+COUNTIF(G52:L52,2)+COUNTIF(G52:L52,3)+COUNTIF(G52:L52,4)+COUNTIF(G52:L52,5),"jen celá čísla 1–5",IF(AND(COUNTA(H52:L52)&gt;0,COUNTA(G52)=0),"doplňte Celkově",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="8" t="inlineStr">
+        <is>
+          <t>T17-B</t>
+        </is>
+      </c>
+      <c r="B53" s="8" t="inlineStr">
+        <is>
+          <t>T17</t>
+        </is>
+      </c>
+      <c r="C53" s="8" t="inlineStr">
+        <is>
+          <t>Farmaceutická fakulta UK v novém kampusu v Hradci Králové: první týdny</t>
+        </is>
+      </c>
+      <c r="D53" s="8" t="inlineStr">
+        <is>
+          <t>Rozšířená rešerše</t>
+        </is>
+      </c>
+      <c r="E53" s="8" t="inlineStr">
+        <is>
+          <t>prošla po jedné opravě</t>
+        </is>
+      </c>
+      <c r="F53" s="8" t="inlineStr">
+        <is>
+          <t>ano</t>
+        </is>
+      </c>
+      <c r="G53" s="8" t="n"/>
+      <c r="H53" s="8" t="n"/>
+      <c r="I53" s="8" t="n"/>
+      <c r="J53" s="8" t="n"/>
+      <c r="K53" s="8" t="n"/>
+      <c r="L53" s="8" t="n"/>
+      <c r="M53" s="8" t="n"/>
+      <c r="N53" s="9">
+        <f>IF(COUNTA(G53:L53)&lt;&gt;COUNTIF(G53:L53,1)+COUNTIF(G53:L53,2)+COUNTIF(G53:L53,3)+COUNTIF(G53:L53,4)+COUNTIF(G53:L53,5),"jen celá čísla 1–5",IF(AND(COUNTA(H53:L53)&gt;0,COUNTA(G53)=0),"doplňte Celkově",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="8" t="inlineStr">
+        <is>
+          <t>T17-C</t>
+        </is>
+      </c>
+      <c r="B54" s="8" t="inlineStr">
+        <is>
+          <t>T17</t>
+        </is>
+      </c>
+      <c r="C54" s="8" t="inlineStr">
+        <is>
+          <t>Farmaceutická fakulta UK v novém kampusu v Hradci Králové: první týdny</t>
+        </is>
+      </c>
+      <c r="D54" s="8" t="inlineStr">
+        <is>
+          <t>Rozšířená rešerše</t>
+        </is>
+      </c>
+      <c r="E54" s="8" t="inlineStr">
+        <is>
+          <t>prošla po jedné opravě</t>
+        </is>
+      </c>
+      <c r="F54" s="8" t="inlineStr">
+        <is>
+          <t>ano</t>
+        </is>
+      </c>
+      <c r="G54" s="8" t="n"/>
+      <c r="H54" s="8" t="n"/>
+      <c r="I54" s="8" t="n"/>
+      <c r="J54" s="8" t="n"/>
+      <c r="K54" s="8" t="n"/>
+      <c r="L54" s="8" t="n"/>
+      <c r="M54" s="8" t="n"/>
+      <c r="N54" s="9">
+        <f>IF(COUNTA(G54:L54)&lt;&gt;COUNTIF(G54:L54,1)+COUNTIF(G54:L54,2)+COUNTIF(G54:L54,3)+COUNTIF(G54:L54,4)+COUNTIF(G54:L54,5),"jen celá čísla 1–5",IF(AND(COUNTA(H54:L54)&gt;0,COUNTA(G54)=0),"doplňte Celkově",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="8" t="inlineStr">
+        <is>
+          <t>T17-D</t>
+        </is>
+      </c>
+      <c r="B55" s="8" t="inlineStr">
+        <is>
+          <t>T17</t>
+        </is>
+      </c>
+      <c r="C55" s="8" t="inlineStr">
+        <is>
+          <t>Farmaceutická fakulta UK v novém kampusu v Hradci Králové: první týdny</t>
+        </is>
+      </c>
+      <c r="D55" s="8" t="inlineStr">
+        <is>
+          <t>Rozšířená rešerše</t>
+        </is>
+      </c>
+      <c r="E55" s="8" t="inlineStr">
+        <is>
+          <t>prošla po jedné opravě</t>
+        </is>
+      </c>
+      <c r="F55" s="8" t="inlineStr">
+        <is>
+          <t>ano</t>
+        </is>
+      </c>
+      <c r="G55" s="8" t="n"/>
+      <c r="H55" s="8" t="n"/>
+      <c r="I55" s="8" t="n"/>
+      <c r="J55" s="8" t="n"/>
+      <c r="K55" s="8" t="n"/>
+      <c r="L55" s="8" t="n"/>
+      <c r="M55" s="8" t="n"/>
+      <c r="N55" s="9">
+        <f>IF(COUNTA(G55:L55)&lt;&gt;COUNTIF(G55:L55,1)+COUNTIF(G55:L55,2)+COUNTIF(G55:L55,3)+COUNTIF(G55:L55,4)+COUNTIF(G55:L55,5),"jen celá čísla 1–5",IF(AND(COUNTA(H55:L55)&gt;0,COUNTA(G55)=0),"doplňte Celkově",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="8" t="inlineStr">
+        <is>
+          <t>T17-E</t>
+        </is>
+      </c>
+      <c r="B56" s="8" t="inlineStr">
+        <is>
+          <t>T17</t>
+        </is>
+      </c>
+      <c r="C56" s="8" t="inlineStr">
+        <is>
+          <t>Farmaceutická fakulta UK v novém kampusu v Hradci Králové: první týdny</t>
+        </is>
+      </c>
+      <c r="D56" s="8" t="inlineStr">
+        <is>
+          <t>Rozšířená rešerše</t>
+        </is>
+      </c>
+      <c r="E56" s="8" t="inlineStr">
+        <is>
+          <t>prošla po jedné opravě</t>
+        </is>
+      </c>
+      <c r="F56" s="8" t="inlineStr">
+        <is>
+          <t>ano</t>
+        </is>
+      </c>
+      <c r="G56" s="8" t="n"/>
+      <c r="H56" s="8" t="n"/>
+      <c r="I56" s="8" t="n"/>
+      <c r="J56" s="8" t="n"/>
+      <c r="K56" s="8" t="n"/>
+      <c r="L56" s="8" t="n"/>
+      <c r="M56" s="8" t="n"/>
+      <c r="N56" s="9">
+        <f>IF(COUNTA(G56:L56)&lt;&gt;COUNTIF(G56:L56,1)+COUNTIF(G56:L56,2)+COUNTIF(G56:L56,3)+COUNTIF(G56:L56,4)+COUNTIF(G56:L56,5),"jen celá čísla 1–5",IF(AND(COUNTA(H56:L56)&gt;0,COUNTA(G56)=0),"doplňte Celkově",""))</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A6:N46"/>
-  <conditionalFormatting sqref="G7:L46">
+  <autoFilter ref="A6:N56"/>
+  <conditionalFormatting sqref="G7:L56">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>IF(G7="",FALSE,IF(ISNUMBER(G7),OR(G7&lt;1,G7&gt;5,G7&lt;&gt;INT(G7)),TRUE))</formula>
     </cfRule>
@@ -2370,11 +2800,11 @@
     <dataValidation sqref="C3" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Hodnotím za" error="Vyberte ze seznamu: VysokeSkoly.cz nebo EffiStream." type="list">
       <formula1>"VysokeSkoly.cz,EffiStream"</formula1>
     </dataValidation>
-    <dataValidation sqref="G8:L8 G9:L9 G10:L10 G11:L11 G12:L12 G15:L15 G16:L16 G17:L17 G19:L19 G20:L20 G21:L21 G22:L22 G23:L23 G24:L24 G26:L26 G30:L30 G31:L31 G33:L33 G34:L34 G35:L35 G36:L36 G37:L37 G38:L38 G39:L39 G40:L40 G41:L41 G42:L42 G43:L43 G44:L44 G45:L45 G46:L46" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Mimo stupnici" error="Zadejte celé číslo 1–5." type="whole" operator="between">
+    <dataValidation sqref="G8:L8 G9:L9 G10:L10 G11:L11 G12:L12 G15:L15 G16:L16 G17:L17 G19:L19 G20:L20 G21:L21 G22:L22 G23:L23 G24:L24 G26:L26 G27:L27 G28:L28 G29:L29 G31:L31 G32:L32 G33:L33 G34:L34 G35:L35 G36:L36 G40:L40 G41:L41 G43:L43 G44:L44 G45:L45 G46:L46 G47:L47 G48:L48 G49:L49 G50:L50 G51:L51 G52:L52 G53:L53 G54:L54 G55:L55 G56:L56" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Mimo stupnici" error="Zadejte celé číslo 1–5." type="whole" operator="between">
       <formula1>1</formula1>
       <formula2>5</formula2>
     </dataValidation>
-    <dataValidation sqref="G7:M7 G13:M13 G14:M14 G18:M18 G25:M25 G27:M27 G28:M28 G29:M29 G32:M32" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Nehodnotí se" error="Tato verze neprošla automatickou kontrolou a nehodnotí se." type="textLength" operator="equal">
+    <dataValidation sqref="G7:M7 G13:M13 G14:M14 G18:M18 G25:M25 G30:M30 G37:M37 G38:M38 G39:M39 G42:M42" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Nehodnotí se" error="Tato verze neprošla automatickou kontrolou a nehodnotí se." type="textLength" operator="equal">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
@@ -2388,7 +2818,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2414,7 +2844,7 @@
         </is>
       </c>
       <c r="B3">
-        <f>COUNTIFS('Hodnocení'!F7:F46,"ano",'Hodnocení'!G7:G46,"&gt;=1",'Hodnocení'!G7:G46,"&lt;=5")</f>
+        <f>COUNTIFS('Hodnocení'!F7:F56,"ano",'Hodnocení'!G7:G56,"&gt;=1",'Hodnocení'!G7:G56,"&lt;=5")</f>
         <v/>
       </c>
     </row>
@@ -2425,7 +2855,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNTIF('Hodnocení'!F7:F46,"ano")</f>
+        <f>COUNTIF('Hodnocení'!F7:F56,"ano")</f>
         <v/>
       </c>
     </row>
@@ -2436,7 +2866,7 @@
         </is>
       </c>
       <c r="B5" s="15">
-        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G46,'Hodnocení'!F7:F46,"ano",'Hodnocení'!G7:G46,"&gt;=1",'Hodnocení'!G7:G46,"&lt;=5"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G56,'Hodnocení'!F7:F56,"ano",'Hodnocení'!G7:G56,"&gt;=1",'Hodnocení'!G7:G56,"&lt;=5"),"")</f>
         <v/>
       </c>
     </row>
@@ -2490,15 +2920,15 @@
         </is>
       </c>
       <c r="D8">
-        <f>COUNTIFS('Hodnocení'!B7:B46,A8,'Hodnocení'!D7:D46,C8,'Hodnocení'!F7:F46,"ano")</f>
+        <f>COUNTIFS('Hodnocení'!B7:B56,A8,'Hodnocení'!D7:D56,C8,'Hodnocení'!F7:F56,"ano")</f>
         <v/>
       </c>
       <c r="E8">
-        <f>COUNTIFS('Hodnocení'!B7:B46,A8,'Hodnocení'!D7:D46,C8,'Hodnocení'!F7:F46,"ano",'Hodnocení'!G7:G46,"&gt;=1",'Hodnocení'!G7:G46,"&lt;=5")</f>
+        <f>COUNTIFS('Hodnocení'!B7:B56,A8,'Hodnocení'!D7:D56,C8,'Hodnocení'!F7:F56,"ano",'Hodnocení'!G7:G56,"&gt;=1",'Hodnocení'!G7:G56,"&lt;=5")</f>
         <v/>
       </c>
       <c r="F8" s="15">
-        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G46,'Hodnocení'!B7:B46,A8,'Hodnocení'!D7:D46,C8,'Hodnocení'!F7:F46,"ano",'Hodnocení'!G7:G46,"&gt;=1",'Hodnocení'!G7:G46,"&lt;=5"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G56,'Hodnocení'!B7:B56,A8,'Hodnocení'!D7:D56,C8,'Hodnocení'!F7:F56,"ano",'Hodnocení'!G7:G56,"&gt;=1",'Hodnocení'!G7:G56,"&lt;=5"),"")</f>
         <v/>
       </c>
     </row>
@@ -2519,15 +2949,15 @@
         </is>
       </c>
       <c r="D9">
-        <f>COUNTIFS('Hodnocení'!B7:B46,A9,'Hodnocení'!D7:D46,C9,'Hodnocení'!F7:F46,"ano")</f>
+        <f>COUNTIFS('Hodnocení'!B7:B56,A9,'Hodnocení'!D7:D56,C9,'Hodnocení'!F7:F56,"ano")</f>
         <v/>
       </c>
       <c r="E9">
-        <f>COUNTIFS('Hodnocení'!B7:B46,A9,'Hodnocení'!D7:D46,C9,'Hodnocení'!F7:F46,"ano",'Hodnocení'!G7:G46,"&gt;=1",'Hodnocení'!G7:G46,"&lt;=5")</f>
+        <f>COUNTIFS('Hodnocení'!B7:B56,A9,'Hodnocení'!D7:D56,C9,'Hodnocení'!F7:F56,"ano",'Hodnocení'!G7:G56,"&gt;=1",'Hodnocení'!G7:G56,"&lt;=5")</f>
         <v/>
       </c>
       <c r="F9" s="15">
-        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G46,'Hodnocení'!B7:B46,A9,'Hodnocení'!D7:D46,C9,'Hodnocení'!F7:F46,"ano",'Hodnocení'!G7:G46,"&gt;=1",'Hodnocení'!G7:G46,"&lt;=5"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G56,'Hodnocení'!B7:B56,A9,'Hodnocení'!D7:D56,C9,'Hodnocení'!F7:F56,"ano",'Hodnocení'!G7:G56,"&gt;=1",'Hodnocení'!G7:G56,"&lt;=5"),"")</f>
         <v/>
       </c>
     </row>
@@ -2548,56 +2978,56 @@
         </is>
       </c>
       <c r="D10">
-        <f>COUNTIFS('Hodnocení'!B7:B46,A10,'Hodnocení'!D7:D46,C10,'Hodnocení'!F7:F46,"ano")</f>
+        <f>COUNTIFS('Hodnocení'!B7:B56,A10,'Hodnocení'!D7:D56,C10,'Hodnocení'!F7:F56,"ano")</f>
         <v/>
       </c>
       <c r="E10">
-        <f>COUNTIFS('Hodnocení'!B7:B46,A10,'Hodnocení'!D7:D46,C10,'Hodnocení'!F7:F46,"ano",'Hodnocení'!G7:G46,"&gt;=1",'Hodnocení'!G7:G46,"&lt;=5")</f>
+        <f>COUNTIFS('Hodnocení'!B7:B56,A10,'Hodnocení'!D7:D56,C10,'Hodnocení'!F7:F56,"ano",'Hodnocení'!G7:G56,"&gt;=1",'Hodnocení'!G7:G56,"&lt;=5")</f>
         <v/>
       </c>
       <c r="F10" s="15">
-        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G46,'Hodnocení'!B7:B46,A10,'Hodnocení'!D7:D46,C10,'Hodnocení'!F7:F46,"ano",'Hodnocení'!G7:G46,"&gt;=1",'Hodnocení'!G7:G46,"&lt;=5"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G56,'Hodnocení'!B7:B56,A10,'Hodnocení'!D7:D56,C10,'Hodnocení'!F7:F56,"ano",'Hodnocení'!G7:G56,"&gt;=1",'Hodnocení'!G7:G56,"&lt;=5"),"")</f>
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>T3</t>
+          <t>T2</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Přestavba strahovských kolejí ČVUT</t>
+          <t>Nový kampus UK v Hradci Králové</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Rozšířená rešerše</t>
+          <t>Automatická cesta</t>
         </is>
       </c>
       <c r="D11">
-        <f>COUNTIFS('Hodnocení'!B7:B46,A11,'Hodnocení'!D7:D46,C11,'Hodnocení'!F7:F46,"ano")</f>
+        <f>COUNTIFS('Hodnocení'!B7:B56,A11,'Hodnocení'!D7:D56,C11,'Hodnocení'!F7:F56,"ano")</f>
         <v/>
       </c>
       <c r="E11">
-        <f>COUNTIFS('Hodnocení'!B7:B46,A11,'Hodnocení'!D7:D46,C11,'Hodnocení'!F7:F46,"ano",'Hodnocení'!G7:G46,"&gt;=1",'Hodnocení'!G7:G46,"&lt;=5")</f>
+        <f>COUNTIFS('Hodnocení'!B7:B56,A11,'Hodnocení'!D7:D56,C11,'Hodnocení'!F7:F56,"ano",'Hodnocení'!G7:G56,"&gt;=1",'Hodnocení'!G7:G56,"&lt;=5")</f>
         <v/>
       </c>
       <c r="F11" s="15">
-        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G46,'Hodnocení'!B7:B46,A11,'Hodnocení'!D7:D46,C11,'Hodnocení'!F7:F46,"ano",'Hodnocení'!G7:G46,"&gt;=1",'Hodnocení'!G7:G46,"&lt;=5"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G56,'Hodnocení'!B7:B56,A11,'Hodnocení'!D7:D56,C11,'Hodnocení'!F7:F56,"ano",'Hodnocení'!G7:G56,"&gt;=1",'Hodnocení'!G7:G56,"&lt;=5"),"")</f>
         <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>T14</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Scio chce založit vlastní vysokou školu</t>
+          <t>Přestavba strahovských kolejí ČVUT</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -2606,27 +3036,27 @@
         </is>
       </c>
       <c r="D12">
-        <f>COUNTIFS('Hodnocení'!B7:B46,A12,'Hodnocení'!D7:D46,C12,'Hodnocení'!F7:F46,"ano")</f>
+        <f>COUNTIFS('Hodnocení'!B7:B56,A12,'Hodnocení'!D7:D56,C12,'Hodnocení'!F7:F56,"ano")</f>
         <v/>
       </c>
       <c r="E12">
-        <f>COUNTIFS('Hodnocení'!B7:B46,A12,'Hodnocení'!D7:D46,C12,'Hodnocení'!F7:F46,"ano",'Hodnocení'!G7:G46,"&gt;=1",'Hodnocení'!G7:G46,"&lt;=5")</f>
+        <f>COUNTIFS('Hodnocení'!B7:B56,A12,'Hodnocení'!D7:D56,C12,'Hodnocení'!F7:F56,"ano",'Hodnocení'!G7:G56,"&gt;=1",'Hodnocení'!G7:G56,"&lt;=5")</f>
         <v/>
       </c>
       <c r="F12" s="15">
-        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G46,'Hodnocení'!B7:B46,A12,'Hodnocení'!D7:D46,C12,'Hodnocení'!F7:F46,"ano",'Hodnocení'!G7:G46,"&gt;=1",'Hodnocení'!G7:G46,"&lt;=5"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G56,'Hodnocení'!B7:B56,A12,'Hodnocení'!D7:D56,C12,'Hodnocení'!F7:F56,"ano",'Hodnocení'!G7:G56,"&gt;=1",'Hodnocení'!G7:G56,"&lt;=5"),"")</f>
         <v/>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>T15</t>
+          <t>T3</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Univerzitní hokejová derby</t>
+          <t>Přestavba strahovských kolejí ČVUT</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2635,27 +3065,27 @@
         </is>
       </c>
       <c r="D13">
-        <f>COUNTIFS('Hodnocení'!B7:B46,A13,'Hodnocení'!D7:D46,C13,'Hodnocení'!F7:F46,"ano")</f>
+        <f>COUNTIFS('Hodnocení'!B7:B56,A13,'Hodnocení'!D7:D56,C13,'Hodnocení'!F7:F56,"ano")</f>
         <v/>
       </c>
       <c r="E13">
-        <f>COUNTIFS('Hodnocení'!B7:B46,A13,'Hodnocení'!D7:D46,C13,'Hodnocení'!F7:F46,"ano",'Hodnocení'!G7:G46,"&gt;=1",'Hodnocení'!G7:G46,"&lt;=5")</f>
+        <f>COUNTIFS('Hodnocení'!B7:B56,A13,'Hodnocení'!D7:D56,C13,'Hodnocení'!F7:F56,"ano",'Hodnocení'!G7:G56,"&gt;=1",'Hodnocení'!G7:G56,"&lt;=5")</f>
         <v/>
       </c>
       <c r="F13" s="15">
-        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G46,'Hodnocení'!B7:B46,A13,'Hodnocení'!D7:D46,C13,'Hodnocení'!F7:F46,"ano",'Hodnocení'!G7:G46,"&gt;=1",'Hodnocení'!G7:G46,"&lt;=5"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G56,'Hodnocení'!B7:B56,A13,'Hodnocení'!D7:D56,C13,'Hodnocení'!F7:F56,"ano",'Hodnocení'!G7:G56,"&gt;=1",'Hodnocení'!G7:G56,"&lt;=5"),"")</f>
         <v/>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>T16</t>
+          <t>T14</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Neúspěch u maturity: jak na další pokus</t>
+          <t>Scio chce založit vlastní vysokou školu</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2664,44 +3094,102 @@
         </is>
       </c>
       <c r="D14">
-        <f>COUNTIFS('Hodnocení'!B7:B46,A14,'Hodnocení'!D7:D46,C14,'Hodnocení'!F7:F46,"ano")</f>
+        <f>COUNTIFS('Hodnocení'!B7:B56,A14,'Hodnocení'!D7:D56,C14,'Hodnocení'!F7:F56,"ano")</f>
         <v/>
       </c>
       <c r="E14">
-        <f>COUNTIFS('Hodnocení'!B7:B46,A14,'Hodnocení'!D7:D46,C14,'Hodnocení'!F7:F46,"ano",'Hodnocení'!G7:G46,"&gt;=1",'Hodnocení'!G7:G46,"&lt;=5")</f>
+        <f>COUNTIFS('Hodnocení'!B7:B56,A14,'Hodnocení'!D7:D56,C14,'Hodnocení'!F7:F56,"ano",'Hodnocení'!G7:G56,"&gt;=1",'Hodnocení'!G7:G56,"&lt;=5")</f>
         <v/>
       </c>
       <c r="F14" s="15">
-        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G46,'Hodnocení'!B7:B46,A14,'Hodnocení'!D7:D46,C14,'Hodnocení'!F7:F46,"ano",'Hodnocení'!G7:G46,"&gt;=1",'Hodnocení'!G7:G46,"&lt;=5"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G56,'Hodnocení'!B7:B56,A14,'Hodnocení'!D7:D56,C14,'Hodnocení'!F7:F56,"ano",'Hodnocení'!G7:G56,"&gt;=1",'Hodnocení'!G7:G56,"&lt;=5"),"")</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>T15</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Univerzitní hokejová derby</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Automatická cesta</t>
+        </is>
+      </c>
+      <c r="D15">
+        <f>COUNTIFS('Hodnocení'!B7:B56,A15,'Hodnocení'!D7:D56,C15,'Hodnocení'!F7:F56,"ano")</f>
+        <v/>
+      </c>
+      <c r="E15">
+        <f>COUNTIFS('Hodnocení'!B7:B56,A15,'Hodnocení'!D7:D56,C15,'Hodnocení'!F7:F56,"ano",'Hodnocení'!G7:G56,"&gt;=1",'Hodnocení'!G7:G56,"&lt;=5")</f>
+        <v/>
+      </c>
+      <c r="F15" s="15">
+        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G56,'Hodnocení'!B7:B56,A15,'Hodnocení'!D7:D56,C15,'Hodnocení'!F7:F56,"ano",'Hodnocení'!G7:G56,"&gt;=1",'Hodnocení'!G7:G56,"&lt;=5"),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>T16</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Neúspěch u maturity: jak na další pokus</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Rozšířená rešerše</t>
+        </is>
+      </c>
+      <c r="D16">
+        <f>COUNTIFS('Hodnocení'!B7:B56,A16,'Hodnocení'!D7:D56,C16,'Hodnocení'!F7:F56,"ano")</f>
+        <v/>
+      </c>
+      <c r="E16">
+        <f>COUNTIFS('Hodnocení'!B7:B56,A16,'Hodnocení'!D7:D56,C16,'Hodnocení'!F7:F56,"ano",'Hodnocení'!G7:G56,"&gt;=1",'Hodnocení'!G7:G56,"&lt;=5")</f>
+        <v/>
+      </c>
+      <c r="F16" s="15">
+        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G56,'Hodnocení'!B7:B56,A16,'Hodnocení'!D7:D56,C16,'Hodnocení'!F7:F56,"ano",'Hodnocení'!G7:G56,"&gt;=1",'Hodnocení'!G7:G56,"&lt;=5"),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>T17</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="B17" t="inlineStr">
         <is>
           <t>Farmaceutická fakulta UK v novém kampusu v Hradci Králové: první týdny</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>Rozšířená rešerše</t>
-        </is>
-      </c>
-      <c r="D15">
-        <f>COUNTIFS('Hodnocení'!B7:B46,A15,'Hodnocení'!D7:D46,C15,'Hodnocení'!F7:F46,"ano")</f>
-        <v/>
-      </c>
-      <c r="E15">
-        <f>COUNTIFS('Hodnocení'!B7:B46,A15,'Hodnocení'!D7:D46,C15,'Hodnocení'!F7:F46,"ano",'Hodnocení'!G7:G46,"&gt;=1",'Hodnocení'!G7:G46,"&lt;=5")</f>
-        <v/>
-      </c>
-      <c r="F15" s="15">
-        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G46,'Hodnocení'!B7:B46,A15,'Hodnocení'!D7:D46,C15,'Hodnocení'!F7:F46,"ano",'Hodnocení'!G7:G46,"&gt;=1",'Hodnocení'!G7:G46,"&lt;=5"),"")</f>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Rozšířená rešerše</t>
+        </is>
+      </c>
+      <c r="D17">
+        <f>COUNTIFS('Hodnocení'!B7:B56,A17,'Hodnocení'!D7:D56,C17,'Hodnocení'!F7:F56,"ano")</f>
+        <v/>
+      </c>
+      <c r="E17">
+        <f>COUNTIFS('Hodnocení'!B7:B56,A17,'Hodnocení'!D7:D56,C17,'Hodnocení'!F7:F56,"ano",'Hodnocení'!G7:G56,"&gt;=1",'Hodnocení'!G7:G56,"&lt;=5")</f>
+        <v/>
+      </c>
+      <c r="F17" s="15">
+        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G56,'Hodnocení'!B7:B56,A17,'Hodnocení'!D7:D56,C17,'Hodnocení'!F7:F56,"ano",'Hodnocení'!G7:G56,"&gt;=1",'Hodnocení'!G7:G56,"&lt;=5"),"")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Automatická cesta: kampus FaF (T17) a maturita (T16) dopsané, podklad k hodnocení 49 verzí
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hodnoceni/hodnoceni-clanku.xlsx
+++ b/hodnoceni/hodnoceni-clanku.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Návod" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Hodnocení'!$A$6:$N$56</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Hodnocení'!$A$6:$N$66</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N56"/>
+  <dimension ref="A1:N66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2577,22 +2577,22 @@
     <row r="52">
       <c r="A52" s="10" t="inlineStr">
         <is>
-          <t>T17-A</t>
+          <t>T16-auto-A</t>
         </is>
       </c>
       <c r="B52" s="10" t="inlineStr">
         <is>
-          <t>T17</t>
+          <t>T16</t>
         </is>
       </c>
       <c r="C52" s="10" t="inlineStr">
         <is>
-          <t>Farmaceutická fakulta UK v novém kampusu v Hradci Králové: první týdny</t>
+          <t>Neúspěch u maturity: jak na další pokus</t>
         </is>
       </c>
       <c r="D52" s="10" t="inlineStr">
         <is>
-          <t>Rozšířená rešerše</t>
+          <t>Automatická cesta</t>
         </is>
       </c>
       <c r="E52" s="10" t="inlineStr">
@@ -2620,22 +2620,22 @@
     <row r="53">
       <c r="A53" s="8" t="inlineStr">
         <is>
-          <t>T17-B</t>
+          <t>T16-auto-B</t>
         </is>
       </c>
       <c r="B53" s="8" t="inlineStr">
         <is>
-          <t>T17</t>
+          <t>T16</t>
         </is>
       </c>
       <c r="C53" s="8" t="inlineStr">
         <is>
-          <t>Farmaceutická fakulta UK v novém kampusu v Hradci Králové: první týdny</t>
+          <t>Neúspěch u maturity: jak na další pokus</t>
         </is>
       </c>
       <c r="D53" s="8" t="inlineStr">
         <is>
-          <t>Rozšířená rešerše</t>
+          <t>Automatická cesta</t>
         </is>
       </c>
       <c r="E53" s="8" t="inlineStr">
@@ -2663,27 +2663,27 @@
     <row r="54">
       <c r="A54" s="8" t="inlineStr">
         <is>
-          <t>T17-C</t>
+          <t>T16-auto-C</t>
         </is>
       </c>
       <c r="B54" s="8" t="inlineStr">
         <is>
-          <t>T17</t>
+          <t>T16</t>
         </is>
       </c>
       <c r="C54" s="8" t="inlineStr">
         <is>
-          <t>Farmaceutická fakulta UK v novém kampusu v Hradci Králové: první týdny</t>
+          <t>Neúspěch u maturity: jak na další pokus</t>
         </is>
       </c>
       <c r="D54" s="8" t="inlineStr">
         <is>
-          <t>Rozšířená rešerše</t>
+          <t>Automatická cesta</t>
         </is>
       </c>
       <c r="E54" s="8" t="inlineStr">
         <is>
-          <t>prošla po jedné opravě</t>
+          <t>prošla napoprvé</t>
         </is>
       </c>
       <c r="F54" s="8" t="inlineStr">
@@ -2706,22 +2706,22 @@
     <row r="55">
       <c r="A55" s="8" t="inlineStr">
         <is>
-          <t>T17-D</t>
+          <t>T16-auto-D</t>
         </is>
       </c>
       <c r="B55" s="8" t="inlineStr">
         <is>
-          <t>T17</t>
+          <t>T16</t>
         </is>
       </c>
       <c r="C55" s="8" t="inlineStr">
         <is>
-          <t>Farmaceutická fakulta UK v novém kampusu v Hradci Králové: první týdny</t>
+          <t>Neúspěch u maturity: jak na další pokus</t>
         </is>
       </c>
       <c r="D55" s="8" t="inlineStr">
         <is>
-          <t>Rozšířená rešerše</t>
+          <t>Automatická cesta</t>
         </is>
       </c>
       <c r="E55" s="8" t="inlineStr">
@@ -2749,27 +2749,27 @@
     <row r="56">
       <c r="A56" s="8" t="inlineStr">
         <is>
-          <t>T17-E</t>
+          <t>T16-auto-E</t>
         </is>
       </c>
       <c r="B56" s="8" t="inlineStr">
         <is>
-          <t>T17</t>
+          <t>T16</t>
         </is>
       </c>
       <c r="C56" s="8" t="inlineStr">
         <is>
-          <t>Farmaceutická fakulta UK v novém kampusu v Hradci Králové: první týdny</t>
+          <t>Neúspěch u maturity: jak na další pokus</t>
         </is>
       </c>
       <c r="D56" s="8" t="inlineStr">
         <is>
-          <t>Rozšířená rešerše</t>
+          <t>Automatická cesta</t>
         </is>
       </c>
       <c r="E56" s="8" t="inlineStr">
         <is>
-          <t>prošla po jedné opravě</t>
+          <t>prošla napoprvé</t>
         </is>
       </c>
       <c r="F56" s="8" t="inlineStr">
@@ -2789,9 +2789,439 @@
         <v/>
       </c>
     </row>
+    <row r="57">
+      <c r="A57" s="10" t="inlineStr">
+        <is>
+          <t>T17-A</t>
+        </is>
+      </c>
+      <c r="B57" s="10" t="inlineStr">
+        <is>
+          <t>T17</t>
+        </is>
+      </c>
+      <c r="C57" s="10" t="inlineStr">
+        <is>
+          <t>Farmaceutická fakulta UK v novém kampusu v Hradci Králové: první týdny</t>
+        </is>
+      </c>
+      <c r="D57" s="10" t="inlineStr">
+        <is>
+          <t>Rozšířená rešerše</t>
+        </is>
+      </c>
+      <c r="E57" s="10" t="inlineStr">
+        <is>
+          <t>prošla napoprvé</t>
+        </is>
+      </c>
+      <c r="F57" s="10" t="inlineStr">
+        <is>
+          <t>ano</t>
+        </is>
+      </c>
+      <c r="G57" s="10" t="n"/>
+      <c r="H57" s="10" t="n"/>
+      <c r="I57" s="10" t="n"/>
+      <c r="J57" s="10" t="n"/>
+      <c r="K57" s="10" t="n"/>
+      <c r="L57" s="10" t="n"/>
+      <c r="M57" s="10" t="n"/>
+      <c r="N57" s="11">
+        <f>IF(COUNTA(G57:L57)&lt;&gt;COUNTIF(G57:L57,1)+COUNTIF(G57:L57,2)+COUNTIF(G57:L57,3)+COUNTIF(G57:L57,4)+COUNTIF(G57:L57,5),"jen celá čísla 1–5",IF(AND(COUNTA(H57:L57)&gt;0,COUNTA(G57)=0),"doplňte Celkově",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="8" t="inlineStr">
+        <is>
+          <t>T17-B</t>
+        </is>
+      </c>
+      <c r="B58" s="8" t="inlineStr">
+        <is>
+          <t>T17</t>
+        </is>
+      </c>
+      <c r="C58" s="8" t="inlineStr">
+        <is>
+          <t>Farmaceutická fakulta UK v novém kampusu v Hradci Králové: první týdny</t>
+        </is>
+      </c>
+      <c r="D58" s="8" t="inlineStr">
+        <is>
+          <t>Rozšířená rešerše</t>
+        </is>
+      </c>
+      <c r="E58" s="8" t="inlineStr">
+        <is>
+          <t>prošla po jedné opravě</t>
+        </is>
+      </c>
+      <c r="F58" s="8" t="inlineStr">
+        <is>
+          <t>ano</t>
+        </is>
+      </c>
+      <c r="G58" s="8" t="n"/>
+      <c r="H58" s="8" t="n"/>
+      <c r="I58" s="8" t="n"/>
+      <c r="J58" s="8" t="n"/>
+      <c r="K58" s="8" t="n"/>
+      <c r="L58" s="8" t="n"/>
+      <c r="M58" s="8" t="n"/>
+      <c r="N58" s="9">
+        <f>IF(COUNTA(G58:L58)&lt;&gt;COUNTIF(G58:L58,1)+COUNTIF(G58:L58,2)+COUNTIF(G58:L58,3)+COUNTIF(G58:L58,4)+COUNTIF(G58:L58,5),"jen celá čísla 1–5",IF(AND(COUNTA(H58:L58)&gt;0,COUNTA(G58)=0),"doplňte Celkově",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="8" t="inlineStr">
+        <is>
+          <t>T17-C</t>
+        </is>
+      </c>
+      <c r="B59" s="8" t="inlineStr">
+        <is>
+          <t>T17</t>
+        </is>
+      </c>
+      <c r="C59" s="8" t="inlineStr">
+        <is>
+          <t>Farmaceutická fakulta UK v novém kampusu v Hradci Králové: první týdny</t>
+        </is>
+      </c>
+      <c r="D59" s="8" t="inlineStr">
+        <is>
+          <t>Rozšířená rešerše</t>
+        </is>
+      </c>
+      <c r="E59" s="8" t="inlineStr">
+        <is>
+          <t>prošla po jedné opravě</t>
+        </is>
+      </c>
+      <c r="F59" s="8" t="inlineStr">
+        <is>
+          <t>ano</t>
+        </is>
+      </c>
+      <c r="G59" s="8" t="n"/>
+      <c r="H59" s="8" t="n"/>
+      <c r="I59" s="8" t="n"/>
+      <c r="J59" s="8" t="n"/>
+      <c r="K59" s="8" t="n"/>
+      <c r="L59" s="8" t="n"/>
+      <c r="M59" s="8" t="n"/>
+      <c r="N59" s="9">
+        <f>IF(COUNTA(G59:L59)&lt;&gt;COUNTIF(G59:L59,1)+COUNTIF(G59:L59,2)+COUNTIF(G59:L59,3)+COUNTIF(G59:L59,4)+COUNTIF(G59:L59,5),"jen celá čísla 1–5",IF(AND(COUNTA(H59:L59)&gt;0,COUNTA(G59)=0),"doplňte Celkově",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="8" t="inlineStr">
+        <is>
+          <t>T17-D</t>
+        </is>
+      </c>
+      <c r="B60" s="8" t="inlineStr">
+        <is>
+          <t>T17</t>
+        </is>
+      </c>
+      <c r="C60" s="8" t="inlineStr">
+        <is>
+          <t>Farmaceutická fakulta UK v novém kampusu v Hradci Králové: první týdny</t>
+        </is>
+      </c>
+      <c r="D60" s="8" t="inlineStr">
+        <is>
+          <t>Rozšířená rešerše</t>
+        </is>
+      </c>
+      <c r="E60" s="8" t="inlineStr">
+        <is>
+          <t>prošla po jedné opravě</t>
+        </is>
+      </c>
+      <c r="F60" s="8" t="inlineStr">
+        <is>
+          <t>ano</t>
+        </is>
+      </c>
+      <c r="G60" s="8" t="n"/>
+      <c r="H60" s="8" t="n"/>
+      <c r="I60" s="8" t="n"/>
+      <c r="J60" s="8" t="n"/>
+      <c r="K60" s="8" t="n"/>
+      <c r="L60" s="8" t="n"/>
+      <c r="M60" s="8" t="n"/>
+      <c r="N60" s="9">
+        <f>IF(COUNTA(G60:L60)&lt;&gt;COUNTIF(G60:L60,1)+COUNTIF(G60:L60,2)+COUNTIF(G60:L60,3)+COUNTIF(G60:L60,4)+COUNTIF(G60:L60,5),"jen celá čísla 1–5",IF(AND(COUNTA(H60:L60)&gt;0,COUNTA(G60)=0),"doplňte Celkově",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="8" t="inlineStr">
+        <is>
+          <t>T17-E</t>
+        </is>
+      </c>
+      <c r="B61" s="8" t="inlineStr">
+        <is>
+          <t>T17</t>
+        </is>
+      </c>
+      <c r="C61" s="8" t="inlineStr">
+        <is>
+          <t>Farmaceutická fakulta UK v novém kampusu v Hradci Králové: první týdny</t>
+        </is>
+      </c>
+      <c r="D61" s="8" t="inlineStr">
+        <is>
+          <t>Rozšířená rešerše</t>
+        </is>
+      </c>
+      <c r="E61" s="8" t="inlineStr">
+        <is>
+          <t>prošla po jedné opravě</t>
+        </is>
+      </c>
+      <c r="F61" s="8" t="inlineStr">
+        <is>
+          <t>ano</t>
+        </is>
+      </c>
+      <c r="G61" s="8" t="n"/>
+      <c r="H61" s="8" t="n"/>
+      <c r="I61" s="8" t="n"/>
+      <c r="J61" s="8" t="n"/>
+      <c r="K61" s="8" t="n"/>
+      <c r="L61" s="8" t="n"/>
+      <c r="M61" s="8" t="n"/>
+      <c r="N61" s="9">
+        <f>IF(COUNTA(G61:L61)&lt;&gt;COUNTIF(G61:L61,1)+COUNTIF(G61:L61,2)+COUNTIF(G61:L61,3)+COUNTIF(G61:L61,4)+COUNTIF(G61:L61,5),"jen celá čísla 1–5",IF(AND(COUNTA(H61:L61)&gt;0,COUNTA(G61)=0),"doplňte Celkově",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="10" t="inlineStr">
+        <is>
+          <t>T17-auto-A</t>
+        </is>
+      </c>
+      <c r="B62" s="10" t="inlineStr">
+        <is>
+          <t>T17</t>
+        </is>
+      </c>
+      <c r="C62" s="10" t="inlineStr">
+        <is>
+          <t>Farmaceutická fakulta UK v novém kampusu v Hradci Králové: první týdny</t>
+        </is>
+      </c>
+      <c r="D62" s="10" t="inlineStr">
+        <is>
+          <t>Automatická cesta</t>
+        </is>
+      </c>
+      <c r="E62" s="10" t="inlineStr">
+        <is>
+          <t>prošla po jedné opravě</t>
+        </is>
+      </c>
+      <c r="F62" s="10" t="inlineStr">
+        <is>
+          <t>ano</t>
+        </is>
+      </c>
+      <c r="G62" s="10" t="n"/>
+      <c r="H62" s="10" t="n"/>
+      <c r="I62" s="10" t="n"/>
+      <c r="J62" s="10" t="n"/>
+      <c r="K62" s="10" t="n"/>
+      <c r="L62" s="10" t="n"/>
+      <c r="M62" s="10" t="n"/>
+      <c r="N62" s="11">
+        <f>IF(COUNTA(G62:L62)&lt;&gt;COUNTIF(G62:L62,1)+COUNTIF(G62:L62,2)+COUNTIF(G62:L62,3)+COUNTIF(G62:L62,4)+COUNTIF(G62:L62,5),"jen celá čísla 1–5",IF(AND(COUNTA(H62:L62)&gt;0,COUNTA(G62)=0),"doplňte Celkově",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="8" t="inlineStr">
+        <is>
+          <t>T17-auto-B</t>
+        </is>
+      </c>
+      <c r="B63" s="8" t="inlineStr">
+        <is>
+          <t>T17</t>
+        </is>
+      </c>
+      <c r="C63" s="8" t="inlineStr">
+        <is>
+          <t>Farmaceutická fakulta UK v novém kampusu v Hradci Králové: první týdny</t>
+        </is>
+      </c>
+      <c r="D63" s="8" t="inlineStr">
+        <is>
+          <t>Automatická cesta</t>
+        </is>
+      </c>
+      <c r="E63" s="8" t="inlineStr">
+        <is>
+          <t>prošla napoprvé</t>
+        </is>
+      </c>
+      <c r="F63" s="8" t="inlineStr">
+        <is>
+          <t>ano</t>
+        </is>
+      </c>
+      <c r="G63" s="8" t="n"/>
+      <c r="H63" s="8" t="n"/>
+      <c r="I63" s="8" t="n"/>
+      <c r="J63" s="8" t="n"/>
+      <c r="K63" s="8" t="n"/>
+      <c r="L63" s="8" t="n"/>
+      <c r="M63" s="8" t="n"/>
+      <c r="N63" s="9">
+        <f>IF(COUNTA(G63:L63)&lt;&gt;COUNTIF(G63:L63,1)+COUNTIF(G63:L63,2)+COUNTIF(G63:L63,3)+COUNTIF(G63:L63,4)+COUNTIF(G63:L63,5),"jen celá čísla 1–5",IF(AND(COUNTA(H63:L63)&gt;0,COUNTA(G63)=0),"doplňte Celkově",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="8" t="inlineStr">
+        <is>
+          <t>T17-auto-C</t>
+        </is>
+      </c>
+      <c r="B64" s="8" t="inlineStr">
+        <is>
+          <t>T17</t>
+        </is>
+      </c>
+      <c r="C64" s="8" t="inlineStr">
+        <is>
+          <t>Farmaceutická fakulta UK v novém kampusu v Hradci Králové: první týdny</t>
+        </is>
+      </c>
+      <c r="D64" s="8" t="inlineStr">
+        <is>
+          <t>Automatická cesta</t>
+        </is>
+      </c>
+      <c r="E64" s="8" t="inlineStr">
+        <is>
+          <t>prošla po jedné opravě</t>
+        </is>
+      </c>
+      <c r="F64" s="8" t="inlineStr">
+        <is>
+          <t>ano</t>
+        </is>
+      </c>
+      <c r="G64" s="8" t="n"/>
+      <c r="H64" s="8" t="n"/>
+      <c r="I64" s="8" t="n"/>
+      <c r="J64" s="8" t="n"/>
+      <c r="K64" s="8" t="n"/>
+      <c r="L64" s="8" t="n"/>
+      <c r="M64" s="8" t="n"/>
+      <c r="N64" s="9">
+        <f>IF(COUNTA(G64:L64)&lt;&gt;COUNTIF(G64:L64,1)+COUNTIF(G64:L64,2)+COUNTIF(G64:L64,3)+COUNTIF(G64:L64,4)+COUNTIF(G64:L64,5),"jen celá čísla 1–5",IF(AND(COUNTA(H64:L64)&gt;0,COUNTA(G64)=0),"doplňte Celkově",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="6" t="inlineStr">
+        <is>
+          <t>T17-auto-D</t>
+        </is>
+      </c>
+      <c r="B65" s="6" t="inlineStr">
+        <is>
+          <t>T17</t>
+        </is>
+      </c>
+      <c r="C65" s="6" t="inlineStr">
+        <is>
+          <t>Farmaceutická fakulta UK v novém kampusu v Hradci Králové: první týdny</t>
+        </is>
+      </c>
+      <c r="D65" s="6" t="inlineStr">
+        <is>
+          <t>Automatická cesta</t>
+        </is>
+      </c>
+      <c r="E65" s="6" t="inlineStr">
+        <is>
+          <t>neprošla – nehodnotí se</t>
+        </is>
+      </c>
+      <c r="F65" s="6" t="inlineStr">
+        <is>
+          <t>ne</t>
+        </is>
+      </c>
+      <c r="G65" s="6" t="n"/>
+      <c r="H65" s="6" t="n"/>
+      <c r="I65" s="6" t="n"/>
+      <c r="J65" s="6" t="n"/>
+      <c r="K65" s="6" t="n"/>
+      <c r="L65" s="6" t="n"/>
+      <c r="M65" s="6" t="n"/>
+      <c r="N65" s="7">
+        <f>IF(COUNTA(G65:L65)&gt;0,"neprošlá verze se nehodnotí","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="8" t="inlineStr">
+        <is>
+          <t>T17-auto-E</t>
+        </is>
+      </c>
+      <c r="B66" s="8" t="inlineStr">
+        <is>
+          <t>T17</t>
+        </is>
+      </c>
+      <c r="C66" s="8" t="inlineStr">
+        <is>
+          <t>Farmaceutická fakulta UK v novém kampusu v Hradci Králové: první týdny</t>
+        </is>
+      </c>
+      <c r="D66" s="8" t="inlineStr">
+        <is>
+          <t>Automatická cesta</t>
+        </is>
+      </c>
+      <c r="E66" s="8" t="inlineStr">
+        <is>
+          <t>prošla po jedné opravě</t>
+        </is>
+      </c>
+      <c r="F66" s="8" t="inlineStr">
+        <is>
+          <t>ano</t>
+        </is>
+      </c>
+      <c r="G66" s="8" t="n"/>
+      <c r="H66" s="8" t="n"/>
+      <c r="I66" s="8" t="n"/>
+      <c r="J66" s="8" t="n"/>
+      <c r="K66" s="8" t="n"/>
+      <c r="L66" s="8" t="n"/>
+      <c r="M66" s="8" t="n"/>
+      <c r="N66" s="9">
+        <f>IF(COUNTA(G66:L66)&lt;&gt;COUNTIF(G66:L66,1)+COUNTIF(G66:L66,2)+COUNTIF(G66:L66,3)+COUNTIF(G66:L66,4)+COUNTIF(G66:L66,5),"jen celá čísla 1–5",IF(AND(COUNTA(H66:L66)&gt;0,COUNTA(G66)=0),"doplňte Celkově",""))</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A6:N56"/>
-  <conditionalFormatting sqref="G7:L56">
+  <autoFilter ref="A6:N66"/>
+  <conditionalFormatting sqref="G7:L66">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>IF(G7="",FALSE,IF(ISNUMBER(G7),OR(G7&lt;1,G7&gt;5,G7&lt;&gt;INT(G7)),TRUE))</formula>
     </cfRule>
@@ -2800,11 +3230,11 @@
     <dataValidation sqref="C3" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Hodnotím za" error="Vyberte ze seznamu: VysokeSkoly.cz nebo EffiStream." type="list">
       <formula1>"VysokeSkoly.cz,EffiStream"</formula1>
     </dataValidation>
-    <dataValidation sqref="G8:L8 G9:L9 G10:L10 G11:L11 G12:L12 G15:L15 G16:L16 G17:L17 G19:L19 G20:L20 G21:L21 G22:L22 G23:L23 G24:L24 G26:L26 G27:L27 G28:L28 G29:L29 G31:L31 G32:L32 G33:L33 G34:L34 G35:L35 G36:L36 G40:L40 G41:L41 G43:L43 G44:L44 G45:L45 G46:L46 G47:L47 G48:L48 G49:L49 G50:L50 G51:L51 G52:L52 G53:L53 G54:L54 G55:L55 G56:L56" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Mimo stupnici" error="Zadejte celé číslo 1–5." type="whole" operator="between">
+    <dataValidation sqref="G8:L8 G9:L9 G10:L10 G11:L11 G12:L12 G15:L15 G16:L16 G17:L17 G19:L19 G20:L20 G21:L21 G22:L22 G23:L23 G24:L24 G26:L26 G27:L27 G28:L28 G29:L29 G31:L31 G32:L32 G33:L33 G34:L34 G35:L35 G36:L36 G40:L40 G41:L41 G43:L43 G44:L44 G45:L45 G46:L46 G47:L47 G48:L48 G49:L49 G50:L50 G51:L51 G52:L52 G53:L53 G54:L54 G55:L55 G56:L56 G57:L57 G58:L58 G59:L59 G60:L60 G61:L61 G62:L62 G63:L63 G64:L64 G66:L66" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Mimo stupnici" error="Zadejte celé číslo 1–5." type="whole" operator="between">
       <formula1>1</formula1>
       <formula2>5</formula2>
     </dataValidation>
-    <dataValidation sqref="G7:M7 G13:M13 G14:M14 G18:M18 G25:M25 G30:M30 G37:M37 G38:M38 G39:M39 G42:M42" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Nehodnotí se" error="Tato verze neprošla automatickou kontrolou a nehodnotí se." type="textLength" operator="equal">
+    <dataValidation sqref="G7:M7 G13:M13 G14:M14 G18:M18 G25:M25 G30:M30 G37:M37 G38:M38 G39:M39 G42:M42 G65:M65" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Nehodnotí se" error="Tato verze neprošla automatickou kontrolou a nehodnotí se." type="textLength" operator="equal">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
@@ -2818,7 +3248,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -2844,7 +3274,7 @@
         </is>
       </c>
       <c r="B3">
-        <f>COUNTIFS('Hodnocení'!F7:F56,"ano",'Hodnocení'!G7:G56,"&gt;=1",'Hodnocení'!G7:G56,"&lt;=5")</f>
+        <f>COUNTIFS('Hodnocení'!F7:F66,"ano",'Hodnocení'!G7:G66,"&gt;=1",'Hodnocení'!G7:G66,"&lt;=5")</f>
         <v/>
       </c>
     </row>
@@ -2855,7 +3285,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNTIF('Hodnocení'!F7:F56,"ano")</f>
+        <f>COUNTIF('Hodnocení'!F7:F66,"ano")</f>
         <v/>
       </c>
     </row>
@@ -2866,7 +3296,7 @@
         </is>
       </c>
       <c r="B5" s="15">
-        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G56,'Hodnocení'!F7:F56,"ano",'Hodnocení'!G7:G56,"&gt;=1",'Hodnocení'!G7:G56,"&lt;=5"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G66,'Hodnocení'!F7:F66,"ano",'Hodnocení'!G7:G66,"&gt;=1",'Hodnocení'!G7:G66,"&lt;=5"),"")</f>
         <v/>
       </c>
     </row>
@@ -2920,15 +3350,15 @@
         </is>
       </c>
       <c r="D8">
-        <f>COUNTIFS('Hodnocení'!B7:B56,A8,'Hodnocení'!D7:D56,C8,'Hodnocení'!F7:F56,"ano")</f>
+        <f>COUNTIFS('Hodnocení'!B7:B66,A8,'Hodnocení'!D7:D66,C8,'Hodnocení'!F7:F66,"ano")</f>
         <v/>
       </c>
       <c r="E8">
-        <f>COUNTIFS('Hodnocení'!B7:B56,A8,'Hodnocení'!D7:D56,C8,'Hodnocení'!F7:F56,"ano",'Hodnocení'!G7:G56,"&gt;=1",'Hodnocení'!G7:G56,"&lt;=5")</f>
+        <f>COUNTIFS('Hodnocení'!B7:B66,A8,'Hodnocení'!D7:D66,C8,'Hodnocení'!F7:F66,"ano",'Hodnocení'!G7:G66,"&gt;=1",'Hodnocení'!G7:G66,"&lt;=5")</f>
         <v/>
       </c>
       <c r="F8" s="15">
-        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G56,'Hodnocení'!B7:B56,A8,'Hodnocení'!D7:D56,C8,'Hodnocení'!F7:F56,"ano",'Hodnocení'!G7:G56,"&gt;=1",'Hodnocení'!G7:G56,"&lt;=5"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G66,'Hodnocení'!B7:B66,A8,'Hodnocení'!D7:D66,C8,'Hodnocení'!F7:F66,"ano",'Hodnocení'!G7:G66,"&gt;=1",'Hodnocení'!G7:G66,"&lt;=5"),"")</f>
         <v/>
       </c>
     </row>
@@ -2949,15 +3379,15 @@
         </is>
       </c>
       <c r="D9">
-        <f>COUNTIFS('Hodnocení'!B7:B56,A9,'Hodnocení'!D7:D56,C9,'Hodnocení'!F7:F56,"ano")</f>
+        <f>COUNTIFS('Hodnocení'!B7:B66,A9,'Hodnocení'!D7:D66,C9,'Hodnocení'!F7:F66,"ano")</f>
         <v/>
       </c>
       <c r="E9">
-        <f>COUNTIFS('Hodnocení'!B7:B56,A9,'Hodnocení'!D7:D56,C9,'Hodnocení'!F7:F56,"ano",'Hodnocení'!G7:G56,"&gt;=1",'Hodnocení'!G7:G56,"&lt;=5")</f>
+        <f>COUNTIFS('Hodnocení'!B7:B66,A9,'Hodnocení'!D7:D66,C9,'Hodnocení'!F7:F66,"ano",'Hodnocení'!G7:G66,"&gt;=1",'Hodnocení'!G7:G66,"&lt;=5")</f>
         <v/>
       </c>
       <c r="F9" s="15">
-        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G56,'Hodnocení'!B7:B56,A9,'Hodnocení'!D7:D56,C9,'Hodnocení'!F7:F56,"ano",'Hodnocení'!G7:G56,"&gt;=1",'Hodnocení'!G7:G56,"&lt;=5"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G66,'Hodnocení'!B7:B66,A9,'Hodnocení'!D7:D66,C9,'Hodnocení'!F7:F66,"ano",'Hodnocení'!G7:G66,"&gt;=1",'Hodnocení'!G7:G66,"&lt;=5"),"")</f>
         <v/>
       </c>
     </row>
@@ -2978,15 +3408,15 @@
         </is>
       </c>
       <c r="D10">
-        <f>COUNTIFS('Hodnocení'!B7:B56,A10,'Hodnocení'!D7:D56,C10,'Hodnocení'!F7:F56,"ano")</f>
+        <f>COUNTIFS('Hodnocení'!B7:B66,A10,'Hodnocení'!D7:D66,C10,'Hodnocení'!F7:F66,"ano")</f>
         <v/>
       </c>
       <c r="E10">
-        <f>COUNTIFS('Hodnocení'!B7:B56,A10,'Hodnocení'!D7:D56,C10,'Hodnocení'!F7:F56,"ano",'Hodnocení'!G7:G56,"&gt;=1",'Hodnocení'!G7:G56,"&lt;=5")</f>
+        <f>COUNTIFS('Hodnocení'!B7:B66,A10,'Hodnocení'!D7:D66,C10,'Hodnocení'!F7:F66,"ano",'Hodnocení'!G7:G66,"&gt;=1",'Hodnocení'!G7:G66,"&lt;=5")</f>
         <v/>
       </c>
       <c r="F10" s="15">
-        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G56,'Hodnocení'!B7:B56,A10,'Hodnocení'!D7:D56,C10,'Hodnocení'!F7:F56,"ano",'Hodnocení'!G7:G56,"&gt;=1",'Hodnocení'!G7:G56,"&lt;=5"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G66,'Hodnocení'!B7:B66,A10,'Hodnocení'!D7:D66,C10,'Hodnocení'!F7:F66,"ano",'Hodnocení'!G7:G66,"&gt;=1",'Hodnocení'!G7:G66,"&lt;=5"),"")</f>
         <v/>
       </c>
     </row>
@@ -3007,15 +3437,15 @@
         </is>
       </c>
       <c r="D11">
-        <f>COUNTIFS('Hodnocení'!B7:B56,A11,'Hodnocení'!D7:D56,C11,'Hodnocení'!F7:F56,"ano")</f>
+        <f>COUNTIFS('Hodnocení'!B7:B66,A11,'Hodnocení'!D7:D66,C11,'Hodnocení'!F7:F66,"ano")</f>
         <v/>
       </c>
       <c r="E11">
-        <f>COUNTIFS('Hodnocení'!B7:B56,A11,'Hodnocení'!D7:D56,C11,'Hodnocení'!F7:F56,"ano",'Hodnocení'!G7:G56,"&gt;=1",'Hodnocení'!G7:G56,"&lt;=5")</f>
+        <f>COUNTIFS('Hodnocení'!B7:B66,A11,'Hodnocení'!D7:D66,C11,'Hodnocení'!F7:F66,"ano",'Hodnocení'!G7:G66,"&gt;=1",'Hodnocení'!G7:G66,"&lt;=5")</f>
         <v/>
       </c>
       <c r="F11" s="15">
-        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G56,'Hodnocení'!B7:B56,A11,'Hodnocení'!D7:D56,C11,'Hodnocení'!F7:F56,"ano",'Hodnocení'!G7:G56,"&gt;=1",'Hodnocení'!G7:G56,"&lt;=5"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G66,'Hodnocení'!B7:B66,A11,'Hodnocení'!D7:D66,C11,'Hodnocení'!F7:F66,"ano",'Hodnocení'!G7:G66,"&gt;=1",'Hodnocení'!G7:G66,"&lt;=5"),"")</f>
         <v/>
       </c>
     </row>
@@ -3036,15 +3466,15 @@
         </is>
       </c>
       <c r="D12">
-        <f>COUNTIFS('Hodnocení'!B7:B56,A12,'Hodnocení'!D7:D56,C12,'Hodnocení'!F7:F56,"ano")</f>
+        <f>COUNTIFS('Hodnocení'!B7:B66,A12,'Hodnocení'!D7:D66,C12,'Hodnocení'!F7:F66,"ano")</f>
         <v/>
       </c>
       <c r="E12">
-        <f>COUNTIFS('Hodnocení'!B7:B56,A12,'Hodnocení'!D7:D56,C12,'Hodnocení'!F7:F56,"ano",'Hodnocení'!G7:G56,"&gt;=1",'Hodnocení'!G7:G56,"&lt;=5")</f>
+        <f>COUNTIFS('Hodnocení'!B7:B66,A12,'Hodnocení'!D7:D66,C12,'Hodnocení'!F7:F66,"ano",'Hodnocení'!G7:G66,"&gt;=1",'Hodnocení'!G7:G66,"&lt;=5")</f>
         <v/>
       </c>
       <c r="F12" s="15">
-        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G56,'Hodnocení'!B7:B56,A12,'Hodnocení'!D7:D56,C12,'Hodnocení'!F7:F56,"ano",'Hodnocení'!G7:G56,"&gt;=1",'Hodnocení'!G7:G56,"&lt;=5"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G66,'Hodnocení'!B7:B66,A12,'Hodnocení'!D7:D66,C12,'Hodnocení'!F7:F66,"ano",'Hodnocení'!G7:G66,"&gt;=1",'Hodnocení'!G7:G66,"&lt;=5"),"")</f>
         <v/>
       </c>
     </row>
@@ -3065,15 +3495,15 @@
         </is>
       </c>
       <c r="D13">
-        <f>COUNTIFS('Hodnocení'!B7:B56,A13,'Hodnocení'!D7:D56,C13,'Hodnocení'!F7:F56,"ano")</f>
+        <f>COUNTIFS('Hodnocení'!B7:B66,A13,'Hodnocení'!D7:D66,C13,'Hodnocení'!F7:F66,"ano")</f>
         <v/>
       </c>
       <c r="E13">
-        <f>COUNTIFS('Hodnocení'!B7:B56,A13,'Hodnocení'!D7:D56,C13,'Hodnocení'!F7:F56,"ano",'Hodnocení'!G7:G56,"&gt;=1",'Hodnocení'!G7:G56,"&lt;=5")</f>
+        <f>COUNTIFS('Hodnocení'!B7:B66,A13,'Hodnocení'!D7:D66,C13,'Hodnocení'!F7:F66,"ano",'Hodnocení'!G7:G66,"&gt;=1",'Hodnocení'!G7:G66,"&lt;=5")</f>
         <v/>
       </c>
       <c r="F13" s="15">
-        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G56,'Hodnocení'!B7:B56,A13,'Hodnocení'!D7:D56,C13,'Hodnocení'!F7:F56,"ano",'Hodnocení'!G7:G56,"&gt;=1",'Hodnocení'!G7:G56,"&lt;=5"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G66,'Hodnocení'!B7:B66,A13,'Hodnocení'!D7:D66,C13,'Hodnocení'!F7:F66,"ano",'Hodnocení'!G7:G66,"&gt;=1",'Hodnocení'!G7:G66,"&lt;=5"),"")</f>
         <v/>
       </c>
     </row>
@@ -3094,15 +3524,15 @@
         </is>
       </c>
       <c r="D14">
-        <f>COUNTIFS('Hodnocení'!B7:B56,A14,'Hodnocení'!D7:D56,C14,'Hodnocení'!F7:F56,"ano")</f>
+        <f>COUNTIFS('Hodnocení'!B7:B66,A14,'Hodnocení'!D7:D66,C14,'Hodnocení'!F7:F66,"ano")</f>
         <v/>
       </c>
       <c r="E14">
-        <f>COUNTIFS('Hodnocení'!B7:B56,A14,'Hodnocení'!D7:D56,C14,'Hodnocení'!F7:F56,"ano",'Hodnocení'!G7:G56,"&gt;=1",'Hodnocení'!G7:G56,"&lt;=5")</f>
+        <f>COUNTIFS('Hodnocení'!B7:B66,A14,'Hodnocení'!D7:D66,C14,'Hodnocení'!F7:F66,"ano",'Hodnocení'!G7:G66,"&gt;=1",'Hodnocení'!G7:G66,"&lt;=5")</f>
         <v/>
       </c>
       <c r="F14" s="15">
-        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G56,'Hodnocení'!B7:B56,A14,'Hodnocení'!D7:D56,C14,'Hodnocení'!F7:F56,"ano",'Hodnocení'!G7:G56,"&gt;=1",'Hodnocení'!G7:G56,"&lt;=5"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G66,'Hodnocení'!B7:B66,A14,'Hodnocení'!D7:D66,C14,'Hodnocení'!F7:F66,"ano",'Hodnocení'!G7:G66,"&gt;=1",'Hodnocení'!G7:G66,"&lt;=5"),"")</f>
         <v/>
       </c>
     </row>
@@ -3123,15 +3553,15 @@
         </is>
       </c>
       <c r="D15">
-        <f>COUNTIFS('Hodnocení'!B7:B56,A15,'Hodnocení'!D7:D56,C15,'Hodnocení'!F7:F56,"ano")</f>
+        <f>COUNTIFS('Hodnocení'!B7:B66,A15,'Hodnocení'!D7:D66,C15,'Hodnocení'!F7:F66,"ano")</f>
         <v/>
       </c>
       <c r="E15">
-        <f>COUNTIFS('Hodnocení'!B7:B56,A15,'Hodnocení'!D7:D56,C15,'Hodnocení'!F7:F56,"ano",'Hodnocení'!G7:G56,"&gt;=1",'Hodnocení'!G7:G56,"&lt;=5")</f>
+        <f>COUNTIFS('Hodnocení'!B7:B66,A15,'Hodnocení'!D7:D66,C15,'Hodnocení'!F7:F66,"ano",'Hodnocení'!G7:G66,"&gt;=1",'Hodnocení'!G7:G66,"&lt;=5")</f>
         <v/>
       </c>
       <c r="F15" s="15">
-        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G56,'Hodnocení'!B7:B56,A15,'Hodnocení'!D7:D56,C15,'Hodnocení'!F7:F56,"ano",'Hodnocení'!G7:G56,"&gt;=1",'Hodnocení'!G7:G56,"&lt;=5"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G66,'Hodnocení'!B7:B66,A15,'Hodnocení'!D7:D66,C15,'Hodnocení'!F7:F66,"ano",'Hodnocení'!G7:G66,"&gt;=1",'Hodnocení'!G7:G66,"&lt;=5"),"")</f>
         <v/>
       </c>
     </row>
@@ -3152,44 +3582,102 @@
         </is>
       </c>
       <c r="D16">
-        <f>COUNTIFS('Hodnocení'!B7:B56,A16,'Hodnocení'!D7:D56,C16,'Hodnocení'!F7:F56,"ano")</f>
+        <f>COUNTIFS('Hodnocení'!B7:B66,A16,'Hodnocení'!D7:D66,C16,'Hodnocení'!F7:F66,"ano")</f>
         <v/>
       </c>
       <c r="E16">
-        <f>COUNTIFS('Hodnocení'!B7:B56,A16,'Hodnocení'!D7:D56,C16,'Hodnocení'!F7:F56,"ano",'Hodnocení'!G7:G56,"&gt;=1",'Hodnocení'!G7:G56,"&lt;=5")</f>
+        <f>COUNTIFS('Hodnocení'!B7:B66,A16,'Hodnocení'!D7:D66,C16,'Hodnocení'!F7:F66,"ano",'Hodnocení'!G7:G66,"&gt;=1",'Hodnocení'!G7:G66,"&lt;=5")</f>
         <v/>
       </c>
       <c r="F16" s="15">
-        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G56,'Hodnocení'!B7:B56,A16,'Hodnocení'!D7:D56,C16,'Hodnocení'!F7:F56,"ano",'Hodnocení'!G7:G56,"&gt;=1",'Hodnocení'!G7:G56,"&lt;=5"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G66,'Hodnocení'!B7:B66,A16,'Hodnocení'!D7:D66,C16,'Hodnocení'!F7:F66,"ano",'Hodnocení'!G7:G66,"&gt;=1",'Hodnocení'!G7:G66,"&lt;=5"),"")</f>
         <v/>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>T16</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Neúspěch u maturity: jak na další pokus</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Automatická cesta</t>
+        </is>
+      </c>
+      <c r="D17">
+        <f>COUNTIFS('Hodnocení'!B7:B66,A17,'Hodnocení'!D7:D66,C17,'Hodnocení'!F7:F66,"ano")</f>
+        <v/>
+      </c>
+      <c r="E17">
+        <f>COUNTIFS('Hodnocení'!B7:B66,A17,'Hodnocení'!D7:D66,C17,'Hodnocení'!F7:F66,"ano",'Hodnocení'!G7:G66,"&gt;=1",'Hodnocení'!G7:G66,"&lt;=5")</f>
+        <v/>
+      </c>
+      <c r="F17" s="15">
+        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G66,'Hodnocení'!B7:B66,A17,'Hodnocení'!D7:D66,C17,'Hodnocení'!F7:F66,"ano",'Hodnocení'!G7:G66,"&gt;=1",'Hodnocení'!G7:G66,"&lt;=5"),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
           <t>T17</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="B18" t="inlineStr">
         <is>
           <t>Farmaceutická fakulta UK v novém kampusu v Hradci Králové: první týdny</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>Rozšířená rešerše</t>
         </is>
       </c>
-      <c r="D17">
-        <f>COUNTIFS('Hodnocení'!B7:B56,A17,'Hodnocení'!D7:D56,C17,'Hodnocení'!F7:F56,"ano")</f>
-        <v/>
-      </c>
-      <c r="E17">
-        <f>COUNTIFS('Hodnocení'!B7:B56,A17,'Hodnocení'!D7:D56,C17,'Hodnocení'!F7:F56,"ano",'Hodnocení'!G7:G56,"&gt;=1",'Hodnocení'!G7:G56,"&lt;=5")</f>
-        <v/>
-      </c>
-      <c r="F17" s="15">
-        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G56,'Hodnocení'!B7:B56,A17,'Hodnocení'!D7:D56,C17,'Hodnocení'!F7:F56,"ano",'Hodnocení'!G7:G56,"&gt;=1",'Hodnocení'!G7:G56,"&lt;=5"),"")</f>
+      <c r="D18">
+        <f>COUNTIFS('Hodnocení'!B7:B66,A18,'Hodnocení'!D7:D66,C18,'Hodnocení'!F7:F66,"ano")</f>
+        <v/>
+      </c>
+      <c r="E18">
+        <f>COUNTIFS('Hodnocení'!B7:B66,A18,'Hodnocení'!D7:D66,C18,'Hodnocení'!F7:F66,"ano",'Hodnocení'!G7:G66,"&gt;=1",'Hodnocení'!G7:G66,"&lt;=5")</f>
+        <v/>
+      </c>
+      <c r="F18" s="15">
+        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G66,'Hodnocení'!B7:B66,A18,'Hodnocení'!D7:D66,C18,'Hodnocení'!F7:F66,"ano",'Hodnocení'!G7:G66,"&gt;=1",'Hodnocení'!G7:G66,"&lt;=5"),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>T17</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Farmaceutická fakulta UK v novém kampusu v Hradci Králové: první týdny</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Automatická cesta</t>
+        </is>
+      </c>
+      <c r="D19">
+        <f>COUNTIFS('Hodnocení'!B7:B66,A19,'Hodnocení'!D7:D66,C19,'Hodnocení'!F7:F66,"ano")</f>
+        <v/>
+      </c>
+      <c r="E19">
+        <f>COUNTIFS('Hodnocení'!B7:B66,A19,'Hodnocení'!D7:D66,C19,'Hodnocení'!F7:F66,"ano",'Hodnocení'!G7:G66,"&gt;=1",'Hodnocení'!G7:G66,"&lt;=5")</f>
+        <v/>
+      </c>
+      <c r="F19" s="15">
+        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G66,'Hodnocení'!B7:B66,A19,'Hodnocení'!D7:D66,C19,'Hodnocení'!F7:F66,"ano",'Hodnocení'!G7:G66,"&gt;=1",'Hodnocení'!G7:G66,"&lt;=5"),"")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
Automatická cesta: Scio (T14) dopsané, podklad k hodnocení 54 verzí
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/hodnoceni/hodnoceni-clanku.xlsx
+++ b/hodnoceni/hodnoceni-clanku.xlsx
@@ -12,7 +12,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Návod" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Hodnocení'!$A$6:$N$66</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Hodnocení'!$A$6:$N$71</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -517,7 +517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N66"/>
+  <dimension ref="A1:N71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2145,62 +2145,62 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="12" t="inlineStr">
-        <is>
-          <t>T15-auto-A</t>
-        </is>
-      </c>
-      <c r="B42" s="12" t="inlineStr">
-        <is>
-          <t>T15</t>
-        </is>
-      </c>
-      <c r="C42" s="12" t="inlineStr">
-        <is>
-          <t>Univerzitní hokejová derby</t>
-        </is>
-      </c>
-      <c r="D42" s="12" t="inlineStr">
+      <c r="A42" s="10" t="inlineStr">
+        <is>
+          <t>T14-auto-A</t>
+        </is>
+      </c>
+      <c r="B42" s="10" t="inlineStr">
+        <is>
+          <t>T14</t>
+        </is>
+      </c>
+      <c r="C42" s="10" t="inlineStr">
+        <is>
+          <t>Scio chce založit vlastní vysokou školu</t>
+        </is>
+      </c>
+      <c r="D42" s="10" t="inlineStr">
         <is>
           <t>Automatická cesta</t>
         </is>
       </c>
-      <c r="E42" s="12" t="inlineStr">
-        <is>
-          <t>neprošla – nehodnotí se</t>
-        </is>
-      </c>
-      <c r="F42" s="12" t="inlineStr">
-        <is>
-          <t>ne</t>
-        </is>
-      </c>
-      <c r="G42" s="12" t="n"/>
-      <c r="H42" s="12" t="n"/>
-      <c r="I42" s="12" t="n"/>
-      <c r="J42" s="12" t="n"/>
-      <c r="K42" s="12" t="n"/>
-      <c r="L42" s="12" t="n"/>
-      <c r="M42" s="12" t="n"/>
-      <c r="N42" s="13">
-        <f>IF(COUNTA(G42:L42)&gt;0,"neprošlá verze se nehodnotí","")</f>
+      <c r="E42" s="10" t="inlineStr">
+        <is>
+          <t>prošla po jedné opravě</t>
+        </is>
+      </c>
+      <c r="F42" s="10" t="inlineStr">
+        <is>
+          <t>ano</t>
+        </is>
+      </c>
+      <c r="G42" s="10" t="n"/>
+      <c r="H42" s="10" t="n"/>
+      <c r="I42" s="10" t="n"/>
+      <c r="J42" s="10" t="n"/>
+      <c r="K42" s="10" t="n"/>
+      <c r="L42" s="10" t="n"/>
+      <c r="M42" s="10" t="n"/>
+      <c r="N42" s="11">
+        <f>IF(COUNTA(G42:L42)&lt;&gt;COUNTIF(G42:L42,1)+COUNTIF(G42:L42,2)+COUNTIF(G42:L42,3)+COUNTIF(G42:L42,4)+COUNTIF(G42:L42,5),"jen celá čísla 1–5",IF(AND(COUNTA(H42:L42)&gt;0,COUNTA(G42)=0),"doplňte Celkově",""))</f>
         <v/>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="8" t="inlineStr">
         <is>
-          <t>T15-auto-B</t>
+          <t>T14-auto-B</t>
         </is>
       </c>
       <c r="B43" s="8" t="inlineStr">
         <is>
-          <t>T15</t>
+          <t>T14</t>
         </is>
       </c>
       <c r="C43" s="8" t="inlineStr">
         <is>
-          <t>Univerzitní hokejová derby</t>
+          <t>Scio chce založit vlastní vysokou školu</t>
         </is>
       </c>
       <c r="D43" s="8" t="inlineStr">
@@ -2233,17 +2233,17 @@
     <row r="44">
       <c r="A44" s="8" t="inlineStr">
         <is>
-          <t>T15-auto-C</t>
+          <t>T14-auto-C</t>
         </is>
       </c>
       <c r="B44" s="8" t="inlineStr">
         <is>
-          <t>T15</t>
+          <t>T14</t>
         </is>
       </c>
       <c r="C44" s="8" t="inlineStr">
         <is>
-          <t>Univerzitní hokejová derby</t>
+          <t>Scio chce založit vlastní vysokou školu</t>
         </is>
       </c>
       <c r="D44" s="8" t="inlineStr">
@@ -2253,7 +2253,7 @@
       </c>
       <c r="E44" s="8" t="inlineStr">
         <is>
-          <t>prošla napoprvé</t>
+          <t>prošla po jedné opravě</t>
         </is>
       </c>
       <c r="F44" s="8" t="inlineStr">
@@ -2276,17 +2276,17 @@
     <row r="45">
       <c r="A45" s="8" t="inlineStr">
         <is>
-          <t>T15-auto-D</t>
+          <t>T14-auto-D</t>
         </is>
       </c>
       <c r="B45" s="8" t="inlineStr">
         <is>
-          <t>T15</t>
+          <t>T14</t>
         </is>
       </c>
       <c r="C45" s="8" t="inlineStr">
         <is>
-          <t>Univerzitní hokejová derby</t>
+          <t>Scio chce založit vlastní vysokou školu</t>
         </is>
       </c>
       <c r="D45" s="8" t="inlineStr">
@@ -2296,7 +2296,7 @@
       </c>
       <c r="E45" s="8" t="inlineStr">
         <is>
-          <t>prošla napoprvé</t>
+          <t>prošla po jedné opravě</t>
         </is>
       </c>
       <c r="F45" s="8" t="inlineStr">
@@ -2319,17 +2319,17 @@
     <row r="46">
       <c r="A46" s="8" t="inlineStr">
         <is>
-          <t>T15-auto-E</t>
+          <t>T14-auto-E</t>
         </is>
       </c>
       <c r="B46" s="8" t="inlineStr">
         <is>
-          <t>T15</t>
+          <t>T14</t>
         </is>
       </c>
       <c r="C46" s="8" t="inlineStr">
         <is>
-          <t>Univerzitní hokejová derby</t>
+          <t>Scio chce založit vlastní vysokou školu</t>
         </is>
       </c>
       <c r="D46" s="8" t="inlineStr">
@@ -2339,7 +2339,7 @@
       </c>
       <c r="E46" s="8" t="inlineStr">
         <is>
-          <t>prošla napoprvé</t>
+          <t>prošla po jedné opravě</t>
         </is>
       </c>
       <c r="F46" s="8" t="inlineStr">
@@ -2360,67 +2360,67 @@
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="10" t="inlineStr">
-        <is>
-          <t>T16-A</t>
-        </is>
-      </c>
-      <c r="B47" s="10" t="inlineStr">
-        <is>
-          <t>T16</t>
-        </is>
-      </c>
-      <c r="C47" s="10" t="inlineStr">
-        <is>
-          <t>Neúspěch u maturity: jak na další pokus</t>
-        </is>
-      </c>
-      <c r="D47" s="10" t="inlineStr">
-        <is>
-          <t>Rozšířená rešerše</t>
-        </is>
-      </c>
-      <c r="E47" s="10" t="inlineStr">
-        <is>
-          <t>prošla napoprvé</t>
-        </is>
-      </c>
-      <c r="F47" s="10" t="inlineStr">
-        <is>
-          <t>ano</t>
-        </is>
-      </c>
-      <c r="G47" s="10" t="n"/>
-      <c r="H47" s="10" t="n"/>
-      <c r="I47" s="10" t="n"/>
-      <c r="J47" s="10" t="n"/>
-      <c r="K47" s="10" t="n"/>
-      <c r="L47" s="10" t="n"/>
-      <c r="M47" s="10" t="n"/>
-      <c r="N47" s="11">
-        <f>IF(COUNTA(G47:L47)&lt;&gt;COUNTIF(G47:L47,1)+COUNTIF(G47:L47,2)+COUNTIF(G47:L47,3)+COUNTIF(G47:L47,4)+COUNTIF(G47:L47,5),"jen celá čísla 1–5",IF(AND(COUNTA(H47:L47)&gt;0,COUNTA(G47)=0),"doplňte Celkově",""))</f>
+      <c r="A47" s="12" t="inlineStr">
+        <is>
+          <t>T15-auto-A</t>
+        </is>
+      </c>
+      <c r="B47" s="12" t="inlineStr">
+        <is>
+          <t>T15</t>
+        </is>
+      </c>
+      <c r="C47" s="12" t="inlineStr">
+        <is>
+          <t>Univerzitní hokejová derby</t>
+        </is>
+      </c>
+      <c r="D47" s="12" t="inlineStr">
+        <is>
+          <t>Automatická cesta</t>
+        </is>
+      </c>
+      <c r="E47" s="12" t="inlineStr">
+        <is>
+          <t>neprošla – nehodnotí se</t>
+        </is>
+      </c>
+      <c r="F47" s="12" t="inlineStr">
+        <is>
+          <t>ne</t>
+        </is>
+      </c>
+      <c r="G47" s="12" t="n"/>
+      <c r="H47" s="12" t="n"/>
+      <c r="I47" s="12" t="n"/>
+      <c r="J47" s="12" t="n"/>
+      <c r="K47" s="12" t="n"/>
+      <c r="L47" s="12" t="n"/>
+      <c r="M47" s="12" t="n"/>
+      <c r="N47" s="13">
+        <f>IF(COUNTA(G47:L47)&gt;0,"neprošlá verze se nehodnotí","")</f>
         <v/>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="8" t="inlineStr">
         <is>
-          <t>T16-B</t>
+          <t>T15-auto-B</t>
         </is>
       </c>
       <c r="B48" s="8" t="inlineStr">
         <is>
-          <t>T16</t>
+          <t>T15</t>
         </is>
       </c>
       <c r="C48" s="8" t="inlineStr">
         <is>
-          <t>Neúspěch u maturity: jak na další pokus</t>
+          <t>Univerzitní hokejová derby</t>
         </is>
       </c>
       <c r="D48" s="8" t="inlineStr">
         <is>
-          <t>Rozšířená rešerše</t>
+          <t>Automatická cesta</t>
         </is>
       </c>
       <c r="E48" s="8" t="inlineStr">
@@ -2448,27 +2448,27 @@
     <row r="49">
       <c r="A49" s="8" t="inlineStr">
         <is>
-          <t>T16-C</t>
+          <t>T15-auto-C</t>
         </is>
       </c>
       <c r="B49" s="8" t="inlineStr">
         <is>
-          <t>T16</t>
+          <t>T15</t>
         </is>
       </c>
       <c r="C49" s="8" t="inlineStr">
         <is>
-          <t>Neúspěch u maturity: jak na další pokus</t>
+          <t>Univerzitní hokejová derby</t>
         </is>
       </c>
       <c r="D49" s="8" t="inlineStr">
         <is>
-          <t>Rozšířená rešerše</t>
+          <t>Automatická cesta</t>
         </is>
       </c>
       <c r="E49" s="8" t="inlineStr">
         <is>
-          <t>prošla po jedné opravě</t>
+          <t>prošla napoprvé</t>
         </is>
       </c>
       <c r="F49" s="8" t="inlineStr">
@@ -2491,27 +2491,27 @@
     <row r="50">
       <c r="A50" s="8" t="inlineStr">
         <is>
-          <t>T16-D</t>
+          <t>T15-auto-D</t>
         </is>
       </c>
       <c r="B50" s="8" t="inlineStr">
         <is>
-          <t>T16</t>
+          <t>T15</t>
         </is>
       </c>
       <c r="C50" s="8" t="inlineStr">
         <is>
-          <t>Neúspěch u maturity: jak na další pokus</t>
+          <t>Univerzitní hokejová derby</t>
         </is>
       </c>
       <c r="D50" s="8" t="inlineStr">
         <is>
-          <t>Rozšířená rešerše</t>
+          <t>Automatická cesta</t>
         </is>
       </c>
       <c r="E50" s="8" t="inlineStr">
         <is>
-          <t>prošla po jedné opravě</t>
+          <t>prošla napoprvé</t>
         </is>
       </c>
       <c r="F50" s="8" t="inlineStr">
@@ -2534,22 +2534,22 @@
     <row r="51">
       <c r="A51" s="8" t="inlineStr">
         <is>
-          <t>T16-E</t>
+          <t>T15-auto-E</t>
         </is>
       </c>
       <c r="B51" s="8" t="inlineStr">
         <is>
-          <t>T16</t>
+          <t>T15</t>
         </is>
       </c>
       <c r="C51" s="8" t="inlineStr">
         <is>
-          <t>Neúspěch u maturity: jak na další pokus</t>
+          <t>Univerzitní hokejová derby</t>
         </is>
       </c>
       <c r="D51" s="8" t="inlineStr">
         <is>
-          <t>Rozšířená rešerše</t>
+          <t>Automatická cesta</t>
         </is>
       </c>
       <c r="E51" s="8" t="inlineStr">
@@ -2577,7 +2577,7 @@
     <row r="52">
       <c r="A52" s="10" t="inlineStr">
         <is>
-          <t>T16-auto-A</t>
+          <t>T16-A</t>
         </is>
       </c>
       <c r="B52" s="10" t="inlineStr">
@@ -2592,7 +2592,7 @@
       </c>
       <c r="D52" s="10" t="inlineStr">
         <is>
-          <t>Automatická cesta</t>
+          <t>Rozšířená rešerše</t>
         </is>
       </c>
       <c r="E52" s="10" t="inlineStr">
@@ -2620,7 +2620,7 @@
     <row r="53">
       <c r="A53" s="8" t="inlineStr">
         <is>
-          <t>T16-auto-B</t>
+          <t>T16-B</t>
         </is>
       </c>
       <c r="B53" s="8" t="inlineStr">
@@ -2635,7 +2635,7 @@
       </c>
       <c r="D53" s="8" t="inlineStr">
         <is>
-          <t>Automatická cesta</t>
+          <t>Rozšířená rešerše</t>
         </is>
       </c>
       <c r="E53" s="8" t="inlineStr">
@@ -2663,7 +2663,7 @@
     <row r="54">
       <c r="A54" s="8" t="inlineStr">
         <is>
-          <t>T16-auto-C</t>
+          <t>T16-C</t>
         </is>
       </c>
       <c r="B54" s="8" t="inlineStr">
@@ -2678,12 +2678,12 @@
       </c>
       <c r="D54" s="8" t="inlineStr">
         <is>
-          <t>Automatická cesta</t>
+          <t>Rozšířená rešerše</t>
         </is>
       </c>
       <c r="E54" s="8" t="inlineStr">
         <is>
-          <t>prošla napoprvé</t>
+          <t>prošla po jedné opravě</t>
         </is>
       </c>
       <c r="F54" s="8" t="inlineStr">
@@ -2706,7 +2706,7 @@
     <row r="55">
       <c r="A55" s="8" t="inlineStr">
         <is>
-          <t>T16-auto-D</t>
+          <t>T16-D</t>
         </is>
       </c>
       <c r="B55" s="8" t="inlineStr">
@@ -2721,7 +2721,7 @@
       </c>
       <c r="D55" s="8" t="inlineStr">
         <is>
-          <t>Automatická cesta</t>
+          <t>Rozšířená rešerše</t>
         </is>
       </c>
       <c r="E55" s="8" t="inlineStr">
@@ -2749,7 +2749,7 @@
     <row r="56">
       <c r="A56" s="8" t="inlineStr">
         <is>
-          <t>T16-auto-E</t>
+          <t>T16-E</t>
         </is>
       </c>
       <c r="B56" s="8" t="inlineStr">
@@ -2764,7 +2764,7 @@
       </c>
       <c r="D56" s="8" t="inlineStr">
         <is>
-          <t>Automatická cesta</t>
+          <t>Rozšířená rešerše</t>
         </is>
       </c>
       <c r="E56" s="8" t="inlineStr">
@@ -2792,22 +2792,22 @@
     <row r="57">
       <c r="A57" s="10" t="inlineStr">
         <is>
-          <t>T17-A</t>
+          <t>T16-auto-A</t>
         </is>
       </c>
       <c r="B57" s="10" t="inlineStr">
         <is>
-          <t>T17</t>
+          <t>T16</t>
         </is>
       </c>
       <c r="C57" s="10" t="inlineStr">
         <is>
-          <t>Farmaceutická fakulta UK v novém kampusu v Hradci Králové: první týdny</t>
+          <t>Neúspěch u maturity: jak na další pokus</t>
         </is>
       </c>
       <c r="D57" s="10" t="inlineStr">
         <is>
-          <t>Rozšířená rešerše</t>
+          <t>Automatická cesta</t>
         </is>
       </c>
       <c r="E57" s="10" t="inlineStr">
@@ -2835,22 +2835,22 @@
     <row r="58">
       <c r="A58" s="8" t="inlineStr">
         <is>
-          <t>T17-B</t>
+          <t>T16-auto-B</t>
         </is>
       </c>
       <c r="B58" s="8" t="inlineStr">
         <is>
-          <t>T17</t>
+          <t>T16</t>
         </is>
       </c>
       <c r="C58" s="8" t="inlineStr">
         <is>
-          <t>Farmaceutická fakulta UK v novém kampusu v Hradci Králové: první týdny</t>
+          <t>Neúspěch u maturity: jak na další pokus</t>
         </is>
       </c>
       <c r="D58" s="8" t="inlineStr">
         <is>
-          <t>Rozšířená rešerše</t>
+          <t>Automatická cesta</t>
         </is>
       </c>
       <c r="E58" s="8" t="inlineStr">
@@ -2878,27 +2878,27 @@
     <row r="59">
       <c r="A59" s="8" t="inlineStr">
         <is>
-          <t>T17-C</t>
+          <t>T16-auto-C</t>
         </is>
       </c>
       <c r="B59" s="8" t="inlineStr">
         <is>
-          <t>T17</t>
+          <t>T16</t>
         </is>
       </c>
       <c r="C59" s="8" t="inlineStr">
         <is>
-          <t>Farmaceutická fakulta UK v novém kampusu v Hradci Králové: první týdny</t>
+          <t>Neúspěch u maturity: jak na další pokus</t>
         </is>
       </c>
       <c r="D59" s="8" t="inlineStr">
         <is>
-          <t>Rozšířená rešerše</t>
+          <t>Automatická cesta</t>
         </is>
       </c>
       <c r="E59" s="8" t="inlineStr">
         <is>
-          <t>prošla po jedné opravě</t>
+          <t>prošla napoprvé</t>
         </is>
       </c>
       <c r="F59" s="8" t="inlineStr">
@@ -2921,22 +2921,22 @@
     <row r="60">
       <c r="A60" s="8" t="inlineStr">
         <is>
-          <t>T17-D</t>
+          <t>T16-auto-D</t>
         </is>
       </c>
       <c r="B60" s="8" t="inlineStr">
         <is>
-          <t>T17</t>
+          <t>T16</t>
         </is>
       </c>
       <c r="C60" s="8" t="inlineStr">
         <is>
-          <t>Farmaceutická fakulta UK v novém kampusu v Hradci Králové: první týdny</t>
+          <t>Neúspěch u maturity: jak na další pokus</t>
         </is>
       </c>
       <c r="D60" s="8" t="inlineStr">
         <is>
-          <t>Rozšířená rešerše</t>
+          <t>Automatická cesta</t>
         </is>
       </c>
       <c r="E60" s="8" t="inlineStr">
@@ -2964,27 +2964,27 @@
     <row r="61">
       <c r="A61" s="8" t="inlineStr">
         <is>
-          <t>T17-E</t>
+          <t>T16-auto-E</t>
         </is>
       </c>
       <c r="B61" s="8" t="inlineStr">
         <is>
-          <t>T17</t>
+          <t>T16</t>
         </is>
       </c>
       <c r="C61" s="8" t="inlineStr">
         <is>
-          <t>Farmaceutická fakulta UK v novém kampusu v Hradci Králové: první týdny</t>
+          <t>Neúspěch u maturity: jak na další pokus</t>
         </is>
       </c>
       <c r="D61" s="8" t="inlineStr">
         <is>
-          <t>Rozšířená rešerše</t>
+          <t>Automatická cesta</t>
         </is>
       </c>
       <c r="E61" s="8" t="inlineStr">
         <is>
-          <t>prošla po jedné opravě</t>
+          <t>prošla napoprvé</t>
         </is>
       </c>
       <c r="F61" s="8" t="inlineStr">
@@ -3007,7 +3007,7 @@
     <row r="62">
       <c r="A62" s="10" t="inlineStr">
         <is>
-          <t>T17-auto-A</t>
+          <t>T17-A</t>
         </is>
       </c>
       <c r="B62" s="10" t="inlineStr">
@@ -3022,12 +3022,12 @@
       </c>
       <c r="D62" s="10" t="inlineStr">
         <is>
-          <t>Automatická cesta</t>
+          <t>Rozšířená rešerše</t>
         </is>
       </c>
       <c r="E62" s="10" t="inlineStr">
         <is>
-          <t>prošla po jedné opravě</t>
+          <t>prošla napoprvé</t>
         </is>
       </c>
       <c r="F62" s="10" t="inlineStr">
@@ -3050,7 +3050,7 @@
     <row r="63">
       <c r="A63" s="8" t="inlineStr">
         <is>
-          <t>T17-auto-B</t>
+          <t>T17-B</t>
         </is>
       </c>
       <c r="B63" s="8" t="inlineStr">
@@ -3065,12 +3065,12 @@
       </c>
       <c r="D63" s="8" t="inlineStr">
         <is>
-          <t>Automatická cesta</t>
+          <t>Rozšířená rešerše</t>
         </is>
       </c>
       <c r="E63" s="8" t="inlineStr">
         <is>
-          <t>prošla napoprvé</t>
+          <t>prošla po jedné opravě</t>
         </is>
       </c>
       <c r="F63" s="8" t="inlineStr">
@@ -3093,7 +3093,7 @@
     <row r="64">
       <c r="A64" s="8" t="inlineStr">
         <is>
-          <t>T17-auto-C</t>
+          <t>T17-C</t>
         </is>
       </c>
       <c r="B64" s="8" t="inlineStr">
@@ -3108,7 +3108,7 @@
       </c>
       <c r="D64" s="8" t="inlineStr">
         <is>
-          <t>Automatická cesta</t>
+          <t>Rozšířená rešerše</t>
         </is>
       </c>
       <c r="E64" s="8" t="inlineStr">
@@ -3134,52 +3134,52 @@
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="6" t="inlineStr">
-        <is>
-          <t>T17-auto-D</t>
-        </is>
-      </c>
-      <c r="B65" s="6" t="inlineStr">
+      <c r="A65" s="8" t="inlineStr">
+        <is>
+          <t>T17-D</t>
+        </is>
+      </c>
+      <c r="B65" s="8" t="inlineStr">
         <is>
           <t>T17</t>
         </is>
       </c>
-      <c r="C65" s="6" t="inlineStr">
+      <c r="C65" s="8" t="inlineStr">
         <is>
           <t>Farmaceutická fakulta UK v novém kampusu v Hradci Králové: první týdny</t>
         </is>
       </c>
-      <c r="D65" s="6" t="inlineStr">
-        <is>
-          <t>Automatická cesta</t>
-        </is>
-      </c>
-      <c r="E65" s="6" t="inlineStr">
-        <is>
-          <t>neprošla – nehodnotí se</t>
-        </is>
-      </c>
-      <c r="F65" s="6" t="inlineStr">
-        <is>
-          <t>ne</t>
-        </is>
-      </c>
-      <c r="G65" s="6" t="n"/>
-      <c r="H65" s="6" t="n"/>
-      <c r="I65" s="6" t="n"/>
-      <c r="J65" s="6" t="n"/>
-      <c r="K65" s="6" t="n"/>
-      <c r="L65" s="6" t="n"/>
-      <c r="M65" s="6" t="n"/>
-      <c r="N65" s="7">
-        <f>IF(COUNTA(G65:L65)&gt;0,"neprošlá verze se nehodnotí","")</f>
+      <c r="D65" s="8" t="inlineStr">
+        <is>
+          <t>Rozšířená rešerše</t>
+        </is>
+      </c>
+      <c r="E65" s="8" t="inlineStr">
+        <is>
+          <t>prošla po jedné opravě</t>
+        </is>
+      </c>
+      <c r="F65" s="8" t="inlineStr">
+        <is>
+          <t>ano</t>
+        </is>
+      </c>
+      <c r="G65" s="8" t="n"/>
+      <c r="H65" s="8" t="n"/>
+      <c r="I65" s="8" t="n"/>
+      <c r="J65" s="8" t="n"/>
+      <c r="K65" s="8" t="n"/>
+      <c r="L65" s="8" t="n"/>
+      <c r="M65" s="8" t="n"/>
+      <c r="N65" s="9">
+        <f>IF(COUNTA(G65:L65)&lt;&gt;COUNTIF(G65:L65,1)+COUNTIF(G65:L65,2)+COUNTIF(G65:L65,3)+COUNTIF(G65:L65,4)+COUNTIF(G65:L65,5),"jen celá čísla 1–5",IF(AND(COUNTA(H65:L65)&gt;0,COUNTA(G65)=0),"doplňte Celkově",""))</f>
         <v/>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="8" t="inlineStr">
         <is>
-          <t>T17-auto-E</t>
+          <t>T17-E</t>
         </is>
       </c>
       <c r="B66" s="8" t="inlineStr">
@@ -3194,7 +3194,7 @@
       </c>
       <c r="D66" s="8" t="inlineStr">
         <is>
-          <t>Automatická cesta</t>
+          <t>Rozšířená rešerše</t>
         </is>
       </c>
       <c r="E66" s="8" t="inlineStr">
@@ -3219,9 +3219,224 @@
         <v/>
       </c>
     </row>
+    <row r="67">
+      <c r="A67" s="10" t="inlineStr">
+        <is>
+          <t>T17-auto-A</t>
+        </is>
+      </c>
+      <c r="B67" s="10" t="inlineStr">
+        <is>
+          <t>T17</t>
+        </is>
+      </c>
+      <c r="C67" s="10" t="inlineStr">
+        <is>
+          <t>Farmaceutická fakulta UK v novém kampusu v Hradci Králové: první týdny</t>
+        </is>
+      </c>
+      <c r="D67" s="10" t="inlineStr">
+        <is>
+          <t>Automatická cesta</t>
+        </is>
+      </c>
+      <c r="E67" s="10" t="inlineStr">
+        <is>
+          <t>prošla po jedné opravě</t>
+        </is>
+      </c>
+      <c r="F67" s="10" t="inlineStr">
+        <is>
+          <t>ano</t>
+        </is>
+      </c>
+      <c r="G67" s="10" t="n"/>
+      <c r="H67" s="10" t="n"/>
+      <c r="I67" s="10" t="n"/>
+      <c r="J67" s="10" t="n"/>
+      <c r="K67" s="10" t="n"/>
+      <c r="L67" s="10" t="n"/>
+      <c r="M67" s="10" t="n"/>
+      <c r="N67" s="11">
+        <f>IF(COUNTA(G67:L67)&lt;&gt;COUNTIF(G67:L67,1)+COUNTIF(G67:L67,2)+COUNTIF(G67:L67,3)+COUNTIF(G67:L67,4)+COUNTIF(G67:L67,5),"jen celá čísla 1–5",IF(AND(COUNTA(H67:L67)&gt;0,COUNTA(G67)=0),"doplňte Celkově",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="8" t="inlineStr">
+        <is>
+          <t>T17-auto-B</t>
+        </is>
+      </c>
+      <c r="B68" s="8" t="inlineStr">
+        <is>
+          <t>T17</t>
+        </is>
+      </c>
+      <c r="C68" s="8" t="inlineStr">
+        <is>
+          <t>Farmaceutická fakulta UK v novém kampusu v Hradci Králové: první týdny</t>
+        </is>
+      </c>
+      <c r="D68" s="8" t="inlineStr">
+        <is>
+          <t>Automatická cesta</t>
+        </is>
+      </c>
+      <c r="E68" s="8" t="inlineStr">
+        <is>
+          <t>prošla napoprvé</t>
+        </is>
+      </c>
+      <c r="F68" s="8" t="inlineStr">
+        <is>
+          <t>ano</t>
+        </is>
+      </c>
+      <c r="G68" s="8" t="n"/>
+      <c r="H68" s="8" t="n"/>
+      <c r="I68" s="8" t="n"/>
+      <c r="J68" s="8" t="n"/>
+      <c r="K68" s="8" t="n"/>
+      <c r="L68" s="8" t="n"/>
+      <c r="M68" s="8" t="n"/>
+      <c r="N68" s="9">
+        <f>IF(COUNTA(G68:L68)&lt;&gt;COUNTIF(G68:L68,1)+COUNTIF(G68:L68,2)+COUNTIF(G68:L68,3)+COUNTIF(G68:L68,4)+COUNTIF(G68:L68,5),"jen celá čísla 1–5",IF(AND(COUNTA(H68:L68)&gt;0,COUNTA(G68)=0),"doplňte Celkově",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="8" t="inlineStr">
+        <is>
+          <t>T17-auto-C</t>
+        </is>
+      </c>
+      <c r="B69" s="8" t="inlineStr">
+        <is>
+          <t>T17</t>
+        </is>
+      </c>
+      <c r="C69" s="8" t="inlineStr">
+        <is>
+          <t>Farmaceutická fakulta UK v novém kampusu v Hradci Králové: první týdny</t>
+        </is>
+      </c>
+      <c r="D69" s="8" t="inlineStr">
+        <is>
+          <t>Automatická cesta</t>
+        </is>
+      </c>
+      <c r="E69" s="8" t="inlineStr">
+        <is>
+          <t>prošla po jedné opravě</t>
+        </is>
+      </c>
+      <c r="F69" s="8" t="inlineStr">
+        <is>
+          <t>ano</t>
+        </is>
+      </c>
+      <c r="G69" s="8" t="n"/>
+      <c r="H69" s="8" t="n"/>
+      <c r="I69" s="8" t="n"/>
+      <c r="J69" s="8" t="n"/>
+      <c r="K69" s="8" t="n"/>
+      <c r="L69" s="8" t="n"/>
+      <c r="M69" s="8" t="n"/>
+      <c r="N69" s="9">
+        <f>IF(COUNTA(G69:L69)&lt;&gt;COUNTIF(G69:L69,1)+COUNTIF(G69:L69,2)+COUNTIF(G69:L69,3)+COUNTIF(G69:L69,4)+COUNTIF(G69:L69,5),"jen celá čísla 1–5",IF(AND(COUNTA(H69:L69)&gt;0,COUNTA(G69)=0),"doplňte Celkově",""))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="6" t="inlineStr">
+        <is>
+          <t>T17-auto-D</t>
+        </is>
+      </c>
+      <c r="B70" s="6" t="inlineStr">
+        <is>
+          <t>T17</t>
+        </is>
+      </c>
+      <c r="C70" s="6" t="inlineStr">
+        <is>
+          <t>Farmaceutická fakulta UK v novém kampusu v Hradci Králové: první týdny</t>
+        </is>
+      </c>
+      <c r="D70" s="6" t="inlineStr">
+        <is>
+          <t>Automatická cesta</t>
+        </is>
+      </c>
+      <c r="E70" s="6" t="inlineStr">
+        <is>
+          <t>neprošla – nehodnotí se</t>
+        </is>
+      </c>
+      <c r="F70" s="6" t="inlineStr">
+        <is>
+          <t>ne</t>
+        </is>
+      </c>
+      <c r="G70" s="6" t="n"/>
+      <c r="H70" s="6" t="n"/>
+      <c r="I70" s="6" t="n"/>
+      <c r="J70" s="6" t="n"/>
+      <c r="K70" s="6" t="n"/>
+      <c r="L70" s="6" t="n"/>
+      <c r="M70" s="6" t="n"/>
+      <c r="N70" s="7">
+        <f>IF(COUNTA(G70:L70)&gt;0,"neprošlá verze se nehodnotí","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="8" t="inlineStr">
+        <is>
+          <t>T17-auto-E</t>
+        </is>
+      </c>
+      <c r="B71" s="8" t="inlineStr">
+        <is>
+          <t>T17</t>
+        </is>
+      </c>
+      <c r="C71" s="8" t="inlineStr">
+        <is>
+          <t>Farmaceutická fakulta UK v novém kampusu v Hradci Králové: první týdny</t>
+        </is>
+      </c>
+      <c r="D71" s="8" t="inlineStr">
+        <is>
+          <t>Automatická cesta</t>
+        </is>
+      </c>
+      <c r="E71" s="8" t="inlineStr">
+        <is>
+          <t>prošla po jedné opravě</t>
+        </is>
+      </c>
+      <c r="F71" s="8" t="inlineStr">
+        <is>
+          <t>ano</t>
+        </is>
+      </c>
+      <c r="G71" s="8" t="n"/>
+      <c r="H71" s="8" t="n"/>
+      <c r="I71" s="8" t="n"/>
+      <c r="J71" s="8" t="n"/>
+      <c r="K71" s="8" t="n"/>
+      <c r="L71" s="8" t="n"/>
+      <c r="M71" s="8" t="n"/>
+      <c r="N71" s="9">
+        <f>IF(COUNTA(G71:L71)&lt;&gt;COUNTIF(G71:L71,1)+COUNTIF(G71:L71,2)+COUNTIF(G71:L71,3)+COUNTIF(G71:L71,4)+COUNTIF(G71:L71,5),"jen celá čísla 1–5",IF(AND(COUNTA(H71:L71)&gt;0,COUNTA(G71)=0),"doplňte Celkově",""))</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A6:N66"/>
-  <conditionalFormatting sqref="G7:L66">
+  <autoFilter ref="A6:N71"/>
+  <conditionalFormatting sqref="G7:L71">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>IF(G7="",FALSE,IF(ISNUMBER(G7),OR(G7&lt;1,G7&gt;5,G7&lt;&gt;INT(G7)),TRUE))</formula>
     </cfRule>
@@ -3230,11 +3445,11 @@
     <dataValidation sqref="C3" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Hodnotím za" error="Vyberte ze seznamu: VysokeSkoly.cz nebo EffiStream." type="list">
       <formula1>"VysokeSkoly.cz,EffiStream"</formula1>
     </dataValidation>
-    <dataValidation sqref="G8:L8 G9:L9 G10:L10 G11:L11 G12:L12 G15:L15 G16:L16 G17:L17 G19:L19 G20:L20 G21:L21 G22:L22 G23:L23 G24:L24 G26:L26 G27:L27 G28:L28 G29:L29 G31:L31 G32:L32 G33:L33 G34:L34 G35:L35 G36:L36 G40:L40 G41:L41 G43:L43 G44:L44 G45:L45 G46:L46 G47:L47 G48:L48 G49:L49 G50:L50 G51:L51 G52:L52 G53:L53 G54:L54 G55:L55 G56:L56 G57:L57 G58:L58 G59:L59 G60:L60 G61:L61 G62:L62 G63:L63 G64:L64 G66:L66" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Mimo stupnici" error="Zadejte celé číslo 1–5." type="whole" operator="between">
+    <dataValidation sqref="G8:L8 G9:L9 G10:L10 G11:L11 G12:L12 G15:L15 G16:L16 G17:L17 G19:L19 G20:L20 G21:L21 G22:L22 G23:L23 G24:L24 G26:L26 G27:L27 G28:L28 G29:L29 G31:L31 G32:L32 G33:L33 G34:L34 G35:L35 G36:L36 G40:L40 G41:L41 G42:L42 G43:L43 G44:L44 G45:L45 G46:L46 G48:L48 G49:L49 G50:L50 G51:L51 G52:L52 G53:L53 G54:L54 G55:L55 G56:L56 G57:L57 G58:L58 G59:L59 G60:L60 G61:L61 G62:L62 G63:L63 G64:L64 G65:L65 G66:L66 G67:L67 G68:L68 G69:L69 G71:L71" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Mimo stupnici" error="Zadejte celé číslo 1–5." type="whole" operator="between">
       <formula1>1</formula1>
       <formula2>5</formula2>
     </dataValidation>
-    <dataValidation sqref="G7:M7 G13:M13 G14:M14 G18:M18 G25:M25 G30:M30 G37:M37 G38:M38 G39:M39 G42:M42 G65:M65" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Nehodnotí se" error="Tato verze neprošla automatickou kontrolou a nehodnotí se." type="textLength" operator="equal">
+    <dataValidation sqref="G7:M7 G13:M13 G14:M14 G18:M18 G25:M25 G30:M30 G37:M37 G38:M38 G39:M39 G47:M47 G70:M70" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Nehodnotí se" error="Tato verze neprošla automatickou kontrolou a nehodnotí se." type="textLength" operator="equal">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>
@@ -3248,7 +3463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:F20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3274,7 +3489,7 @@
         </is>
       </c>
       <c r="B3">
-        <f>COUNTIFS('Hodnocení'!F7:F66,"ano",'Hodnocení'!G7:G66,"&gt;=1",'Hodnocení'!G7:G66,"&lt;=5")</f>
+        <f>COUNTIFS('Hodnocení'!F7:F71,"ano",'Hodnocení'!G7:G71,"&gt;=1",'Hodnocení'!G7:G71,"&lt;=5")</f>
         <v/>
       </c>
     </row>
@@ -3285,7 +3500,7 @@
         </is>
       </c>
       <c r="B4">
-        <f>COUNTIF('Hodnocení'!F7:F66,"ano")</f>
+        <f>COUNTIF('Hodnocení'!F7:F71,"ano")</f>
         <v/>
       </c>
     </row>
@@ -3296,7 +3511,7 @@
         </is>
       </c>
       <c r="B5" s="15">
-        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G66,'Hodnocení'!F7:F66,"ano",'Hodnocení'!G7:G66,"&gt;=1",'Hodnocení'!G7:G66,"&lt;=5"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G71,'Hodnocení'!F7:F71,"ano",'Hodnocení'!G7:G71,"&gt;=1",'Hodnocení'!G7:G71,"&lt;=5"),"")</f>
         <v/>
       </c>
     </row>
@@ -3350,15 +3565,15 @@
         </is>
       </c>
       <c r="D8">
-        <f>COUNTIFS('Hodnocení'!B7:B66,A8,'Hodnocení'!D7:D66,C8,'Hodnocení'!F7:F66,"ano")</f>
+        <f>COUNTIFS('Hodnocení'!B7:B71,A8,'Hodnocení'!D7:D71,C8,'Hodnocení'!F7:F71,"ano")</f>
         <v/>
       </c>
       <c r="E8">
-        <f>COUNTIFS('Hodnocení'!B7:B66,A8,'Hodnocení'!D7:D66,C8,'Hodnocení'!F7:F66,"ano",'Hodnocení'!G7:G66,"&gt;=1",'Hodnocení'!G7:G66,"&lt;=5")</f>
+        <f>COUNTIFS('Hodnocení'!B7:B71,A8,'Hodnocení'!D7:D71,C8,'Hodnocení'!F7:F71,"ano",'Hodnocení'!G7:G71,"&gt;=1",'Hodnocení'!G7:G71,"&lt;=5")</f>
         <v/>
       </c>
       <c r="F8" s="15">
-        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G66,'Hodnocení'!B7:B66,A8,'Hodnocení'!D7:D66,C8,'Hodnocení'!F7:F66,"ano",'Hodnocení'!G7:G66,"&gt;=1",'Hodnocení'!G7:G66,"&lt;=5"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G71,'Hodnocení'!B7:B71,A8,'Hodnocení'!D7:D71,C8,'Hodnocení'!F7:F71,"ano",'Hodnocení'!G7:G71,"&gt;=1",'Hodnocení'!G7:G71,"&lt;=5"),"")</f>
         <v/>
       </c>
     </row>
@@ -3379,15 +3594,15 @@
         </is>
       </c>
       <c r="D9">
-        <f>COUNTIFS('Hodnocení'!B7:B66,A9,'Hodnocení'!D7:D66,C9,'Hodnocení'!F7:F66,"ano")</f>
+        <f>COUNTIFS('Hodnocení'!B7:B71,A9,'Hodnocení'!D7:D71,C9,'Hodnocení'!F7:F71,"ano")</f>
         <v/>
       </c>
       <c r="E9">
-        <f>COUNTIFS('Hodnocení'!B7:B66,A9,'Hodnocení'!D7:D66,C9,'Hodnocení'!F7:F66,"ano",'Hodnocení'!G7:G66,"&gt;=1",'Hodnocení'!G7:G66,"&lt;=5")</f>
+        <f>COUNTIFS('Hodnocení'!B7:B71,A9,'Hodnocení'!D7:D71,C9,'Hodnocení'!F7:F71,"ano",'Hodnocení'!G7:G71,"&gt;=1",'Hodnocení'!G7:G71,"&lt;=5")</f>
         <v/>
       </c>
       <c r="F9" s="15">
-        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G66,'Hodnocení'!B7:B66,A9,'Hodnocení'!D7:D66,C9,'Hodnocení'!F7:F66,"ano",'Hodnocení'!G7:G66,"&gt;=1",'Hodnocení'!G7:G66,"&lt;=5"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G71,'Hodnocení'!B7:B71,A9,'Hodnocení'!D7:D71,C9,'Hodnocení'!F7:F71,"ano",'Hodnocení'!G7:G71,"&gt;=1",'Hodnocení'!G7:G71,"&lt;=5"),"")</f>
         <v/>
       </c>
     </row>
@@ -3408,15 +3623,15 @@
         </is>
       </c>
       <c r="D10">
-        <f>COUNTIFS('Hodnocení'!B7:B66,A10,'Hodnocení'!D7:D66,C10,'Hodnocení'!F7:F66,"ano")</f>
+        <f>COUNTIFS('Hodnocení'!B7:B71,A10,'Hodnocení'!D7:D71,C10,'Hodnocení'!F7:F71,"ano")</f>
         <v/>
       </c>
       <c r="E10">
-        <f>COUNTIFS('Hodnocení'!B7:B66,A10,'Hodnocení'!D7:D66,C10,'Hodnocení'!F7:F66,"ano",'Hodnocení'!G7:G66,"&gt;=1",'Hodnocení'!G7:G66,"&lt;=5")</f>
+        <f>COUNTIFS('Hodnocení'!B7:B71,A10,'Hodnocení'!D7:D71,C10,'Hodnocení'!F7:F71,"ano",'Hodnocení'!G7:G71,"&gt;=1",'Hodnocení'!G7:G71,"&lt;=5")</f>
         <v/>
       </c>
       <c r="F10" s="15">
-        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G66,'Hodnocení'!B7:B66,A10,'Hodnocení'!D7:D66,C10,'Hodnocení'!F7:F66,"ano",'Hodnocení'!G7:G66,"&gt;=1",'Hodnocení'!G7:G66,"&lt;=5"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G71,'Hodnocení'!B7:B71,A10,'Hodnocení'!D7:D71,C10,'Hodnocení'!F7:F71,"ano",'Hodnocení'!G7:G71,"&gt;=1",'Hodnocení'!G7:G71,"&lt;=5"),"")</f>
         <v/>
       </c>
     </row>
@@ -3437,15 +3652,15 @@
         </is>
       </c>
       <c r="D11">
-        <f>COUNTIFS('Hodnocení'!B7:B66,A11,'Hodnocení'!D7:D66,C11,'Hodnocení'!F7:F66,"ano")</f>
+        <f>COUNTIFS('Hodnocení'!B7:B71,A11,'Hodnocení'!D7:D71,C11,'Hodnocení'!F7:F71,"ano")</f>
         <v/>
       </c>
       <c r="E11">
-        <f>COUNTIFS('Hodnocení'!B7:B66,A11,'Hodnocení'!D7:D66,C11,'Hodnocení'!F7:F66,"ano",'Hodnocení'!G7:G66,"&gt;=1",'Hodnocení'!G7:G66,"&lt;=5")</f>
+        <f>COUNTIFS('Hodnocení'!B7:B71,A11,'Hodnocení'!D7:D71,C11,'Hodnocení'!F7:F71,"ano",'Hodnocení'!G7:G71,"&gt;=1",'Hodnocení'!G7:G71,"&lt;=5")</f>
         <v/>
       </c>
       <c r="F11" s="15">
-        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G66,'Hodnocení'!B7:B66,A11,'Hodnocení'!D7:D66,C11,'Hodnocení'!F7:F66,"ano",'Hodnocení'!G7:G66,"&gt;=1",'Hodnocení'!G7:G66,"&lt;=5"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G71,'Hodnocení'!B7:B71,A11,'Hodnocení'!D7:D71,C11,'Hodnocení'!F7:F71,"ano",'Hodnocení'!G7:G71,"&gt;=1",'Hodnocení'!G7:G71,"&lt;=5"),"")</f>
         <v/>
       </c>
     </row>
@@ -3466,15 +3681,15 @@
         </is>
       </c>
       <c r="D12">
-        <f>COUNTIFS('Hodnocení'!B7:B66,A12,'Hodnocení'!D7:D66,C12,'Hodnocení'!F7:F66,"ano")</f>
+        <f>COUNTIFS('Hodnocení'!B7:B71,A12,'Hodnocení'!D7:D71,C12,'Hodnocení'!F7:F71,"ano")</f>
         <v/>
       </c>
       <c r="E12">
-        <f>COUNTIFS('Hodnocení'!B7:B66,A12,'Hodnocení'!D7:D66,C12,'Hodnocení'!F7:F66,"ano",'Hodnocení'!G7:G66,"&gt;=1",'Hodnocení'!G7:G66,"&lt;=5")</f>
+        <f>COUNTIFS('Hodnocení'!B7:B71,A12,'Hodnocení'!D7:D71,C12,'Hodnocení'!F7:F71,"ano",'Hodnocení'!G7:G71,"&gt;=1",'Hodnocení'!G7:G71,"&lt;=5")</f>
         <v/>
       </c>
       <c r="F12" s="15">
-        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G66,'Hodnocení'!B7:B66,A12,'Hodnocení'!D7:D66,C12,'Hodnocení'!F7:F66,"ano",'Hodnocení'!G7:G66,"&gt;=1",'Hodnocení'!G7:G66,"&lt;=5"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G71,'Hodnocení'!B7:B71,A12,'Hodnocení'!D7:D71,C12,'Hodnocení'!F7:F71,"ano",'Hodnocení'!G7:G71,"&gt;=1",'Hodnocení'!G7:G71,"&lt;=5"),"")</f>
         <v/>
       </c>
     </row>
@@ -3495,15 +3710,15 @@
         </is>
       </c>
       <c r="D13">
-        <f>COUNTIFS('Hodnocení'!B7:B66,A13,'Hodnocení'!D7:D66,C13,'Hodnocení'!F7:F66,"ano")</f>
+        <f>COUNTIFS('Hodnocení'!B7:B71,A13,'Hodnocení'!D7:D71,C13,'Hodnocení'!F7:F71,"ano")</f>
         <v/>
       </c>
       <c r="E13">
-        <f>COUNTIFS('Hodnocení'!B7:B66,A13,'Hodnocení'!D7:D66,C13,'Hodnocení'!F7:F66,"ano",'Hodnocení'!G7:G66,"&gt;=1",'Hodnocení'!G7:G66,"&lt;=5")</f>
+        <f>COUNTIFS('Hodnocení'!B7:B71,A13,'Hodnocení'!D7:D71,C13,'Hodnocení'!F7:F71,"ano",'Hodnocení'!G7:G71,"&gt;=1",'Hodnocení'!G7:G71,"&lt;=5")</f>
         <v/>
       </c>
       <c r="F13" s="15">
-        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G66,'Hodnocení'!B7:B66,A13,'Hodnocení'!D7:D66,C13,'Hodnocení'!F7:F66,"ano",'Hodnocení'!G7:G66,"&gt;=1",'Hodnocení'!G7:G66,"&lt;=5"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G71,'Hodnocení'!B7:B71,A13,'Hodnocení'!D7:D71,C13,'Hodnocení'!F7:F71,"ano",'Hodnocení'!G7:G71,"&gt;=1",'Hodnocení'!G7:G71,"&lt;=5"),"")</f>
         <v/>
       </c>
     </row>
@@ -3524,27 +3739,27 @@
         </is>
       </c>
       <c r="D14">
-        <f>COUNTIFS('Hodnocení'!B7:B66,A14,'Hodnocení'!D7:D66,C14,'Hodnocení'!F7:F66,"ano")</f>
+        <f>COUNTIFS('Hodnocení'!B7:B71,A14,'Hodnocení'!D7:D71,C14,'Hodnocení'!F7:F71,"ano")</f>
         <v/>
       </c>
       <c r="E14">
-        <f>COUNTIFS('Hodnocení'!B7:B66,A14,'Hodnocení'!D7:D66,C14,'Hodnocení'!F7:F66,"ano",'Hodnocení'!G7:G66,"&gt;=1",'Hodnocení'!G7:G66,"&lt;=5")</f>
+        <f>COUNTIFS('Hodnocení'!B7:B71,A14,'Hodnocení'!D7:D71,C14,'Hodnocení'!F7:F71,"ano",'Hodnocení'!G7:G71,"&gt;=1",'Hodnocení'!G7:G71,"&lt;=5")</f>
         <v/>
       </c>
       <c r="F14" s="15">
-        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G66,'Hodnocení'!B7:B66,A14,'Hodnocení'!D7:D66,C14,'Hodnocení'!F7:F66,"ano",'Hodnocení'!G7:G66,"&gt;=1",'Hodnocení'!G7:G66,"&lt;=5"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G71,'Hodnocení'!B7:B71,A14,'Hodnocení'!D7:D71,C14,'Hodnocení'!F7:F71,"ano",'Hodnocení'!G7:G71,"&gt;=1",'Hodnocení'!G7:G71,"&lt;=5"),"")</f>
         <v/>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>T15</t>
+          <t>T14</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Univerzitní hokejová derby</t>
+          <t>Scio chce založit vlastní vysokou školu</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -3553,44 +3768,44 @@
         </is>
       </c>
       <c r="D15">
-        <f>COUNTIFS('Hodnocení'!B7:B66,A15,'Hodnocení'!D7:D66,C15,'Hodnocení'!F7:F66,"ano")</f>
+        <f>COUNTIFS('Hodnocení'!B7:B71,A15,'Hodnocení'!D7:D71,C15,'Hodnocení'!F7:F71,"ano")</f>
         <v/>
       </c>
       <c r="E15">
-        <f>COUNTIFS('Hodnocení'!B7:B66,A15,'Hodnocení'!D7:D66,C15,'Hodnocení'!F7:F66,"ano",'Hodnocení'!G7:G66,"&gt;=1",'Hodnocení'!G7:G66,"&lt;=5")</f>
+        <f>COUNTIFS('Hodnocení'!B7:B71,A15,'Hodnocení'!D7:D71,C15,'Hodnocení'!F7:F71,"ano",'Hodnocení'!G7:G71,"&gt;=1",'Hodnocení'!G7:G71,"&lt;=5")</f>
         <v/>
       </c>
       <c r="F15" s="15">
-        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G66,'Hodnocení'!B7:B66,A15,'Hodnocení'!D7:D66,C15,'Hodnocení'!F7:F66,"ano",'Hodnocení'!G7:G66,"&gt;=1",'Hodnocení'!G7:G66,"&lt;=5"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G71,'Hodnocení'!B7:B71,A15,'Hodnocení'!D7:D71,C15,'Hodnocení'!F7:F71,"ano",'Hodnocení'!G7:G71,"&gt;=1",'Hodnocení'!G7:G71,"&lt;=5"),"")</f>
         <v/>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>T16</t>
+          <t>T15</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Neúspěch u maturity: jak na další pokus</t>
+          <t>Univerzitní hokejová derby</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Rozšířená rešerše</t>
+          <t>Automatická cesta</t>
         </is>
       </c>
       <c r="D16">
-        <f>COUNTIFS('Hodnocení'!B7:B66,A16,'Hodnocení'!D7:D66,C16,'Hodnocení'!F7:F66,"ano")</f>
+        <f>COUNTIFS('Hodnocení'!B7:B71,A16,'Hodnocení'!D7:D71,C16,'Hodnocení'!F7:F71,"ano")</f>
         <v/>
       </c>
       <c r="E16">
-        <f>COUNTIFS('Hodnocení'!B7:B66,A16,'Hodnocení'!D7:D66,C16,'Hodnocení'!F7:F66,"ano",'Hodnocení'!G7:G66,"&gt;=1",'Hodnocení'!G7:G66,"&lt;=5")</f>
+        <f>COUNTIFS('Hodnocení'!B7:B71,A16,'Hodnocení'!D7:D71,C16,'Hodnocení'!F7:F71,"ano",'Hodnocení'!G7:G71,"&gt;=1",'Hodnocení'!G7:G71,"&lt;=5")</f>
         <v/>
       </c>
       <c r="F16" s="15">
-        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G66,'Hodnocení'!B7:B66,A16,'Hodnocení'!D7:D66,C16,'Hodnocení'!F7:F66,"ano",'Hodnocení'!G7:G66,"&gt;=1",'Hodnocení'!G7:G66,"&lt;=5"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G71,'Hodnocení'!B7:B71,A16,'Hodnocení'!D7:D71,C16,'Hodnocení'!F7:F71,"ano",'Hodnocení'!G7:G71,"&gt;=1",'Hodnocení'!G7:G71,"&lt;=5"),"")</f>
         <v/>
       </c>
     </row>
@@ -3607,48 +3822,48 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Automatická cesta</t>
+          <t>Rozšířená rešerše</t>
         </is>
       </c>
       <c r="D17">
-        <f>COUNTIFS('Hodnocení'!B7:B66,A17,'Hodnocení'!D7:D66,C17,'Hodnocení'!F7:F66,"ano")</f>
+        <f>COUNTIFS('Hodnocení'!B7:B71,A17,'Hodnocení'!D7:D71,C17,'Hodnocení'!F7:F71,"ano")</f>
         <v/>
       </c>
       <c r="E17">
-        <f>COUNTIFS('Hodnocení'!B7:B66,A17,'Hodnocení'!D7:D66,C17,'Hodnocení'!F7:F66,"ano",'Hodnocení'!G7:G66,"&gt;=1",'Hodnocení'!G7:G66,"&lt;=5")</f>
+        <f>COUNTIFS('Hodnocení'!B7:B71,A17,'Hodnocení'!D7:D71,C17,'Hodnocení'!F7:F71,"ano",'Hodnocení'!G7:G71,"&gt;=1",'Hodnocení'!G7:G71,"&lt;=5")</f>
         <v/>
       </c>
       <c r="F17" s="15">
-        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G66,'Hodnocení'!B7:B66,A17,'Hodnocení'!D7:D66,C17,'Hodnocení'!F7:F66,"ano",'Hodnocení'!G7:G66,"&gt;=1",'Hodnocení'!G7:G66,"&lt;=5"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G71,'Hodnocení'!B7:B71,A17,'Hodnocení'!D7:D71,C17,'Hodnocení'!F7:F71,"ano",'Hodnocení'!G7:G71,"&gt;=1",'Hodnocení'!G7:G71,"&lt;=5"),"")</f>
         <v/>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>T17</t>
+          <t>T16</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Farmaceutická fakulta UK v novém kampusu v Hradci Králové: první týdny</t>
+          <t>Neúspěch u maturity: jak na další pokus</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Rozšířená rešerše</t>
+          <t>Automatická cesta</t>
         </is>
       </c>
       <c r="D18">
-        <f>COUNTIFS('Hodnocení'!B7:B66,A18,'Hodnocení'!D7:D66,C18,'Hodnocení'!F7:F66,"ano")</f>
+        <f>COUNTIFS('Hodnocení'!B7:B71,A18,'Hodnocení'!D7:D71,C18,'Hodnocení'!F7:F71,"ano")</f>
         <v/>
       </c>
       <c r="E18">
-        <f>COUNTIFS('Hodnocení'!B7:B66,A18,'Hodnocení'!D7:D66,C18,'Hodnocení'!F7:F66,"ano",'Hodnocení'!G7:G66,"&gt;=1",'Hodnocení'!G7:G66,"&lt;=5")</f>
+        <f>COUNTIFS('Hodnocení'!B7:B71,A18,'Hodnocení'!D7:D71,C18,'Hodnocení'!F7:F71,"ano",'Hodnocení'!G7:G71,"&gt;=1",'Hodnocení'!G7:G71,"&lt;=5")</f>
         <v/>
       </c>
       <c r="F18" s="15">
-        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G66,'Hodnocení'!B7:B66,A18,'Hodnocení'!D7:D66,C18,'Hodnocení'!F7:F66,"ano",'Hodnocení'!G7:G66,"&gt;=1",'Hodnocení'!G7:G66,"&lt;=5"),"")</f>
+        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G71,'Hodnocení'!B7:B71,A18,'Hodnocení'!D7:D71,C18,'Hodnocení'!F7:F71,"ano",'Hodnocení'!G7:G71,"&gt;=1",'Hodnocení'!G7:G71,"&lt;=5"),"")</f>
         <v/>
       </c>
     </row>
@@ -3665,19 +3880,48 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
+          <t>Rozšířená rešerše</t>
+        </is>
+      </c>
+      <c r="D19">
+        <f>COUNTIFS('Hodnocení'!B7:B71,A19,'Hodnocení'!D7:D71,C19,'Hodnocení'!F7:F71,"ano")</f>
+        <v/>
+      </c>
+      <c r="E19">
+        <f>COUNTIFS('Hodnocení'!B7:B71,A19,'Hodnocení'!D7:D71,C19,'Hodnocení'!F7:F71,"ano",'Hodnocení'!G7:G71,"&gt;=1",'Hodnocení'!G7:G71,"&lt;=5")</f>
+        <v/>
+      </c>
+      <c r="F19" s="15">
+        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G71,'Hodnocení'!B7:B71,A19,'Hodnocení'!D7:D71,C19,'Hodnocení'!F7:F71,"ano",'Hodnocení'!G7:G71,"&gt;=1",'Hodnocení'!G7:G71,"&lt;=5"),"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>T17</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Farmaceutická fakulta UK v novém kampusu v Hradci Králové: první týdny</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
           <t>Automatická cesta</t>
         </is>
       </c>
-      <c r="D19">
-        <f>COUNTIFS('Hodnocení'!B7:B66,A19,'Hodnocení'!D7:D66,C19,'Hodnocení'!F7:F66,"ano")</f>
-        <v/>
-      </c>
-      <c r="E19">
-        <f>COUNTIFS('Hodnocení'!B7:B66,A19,'Hodnocení'!D7:D66,C19,'Hodnocení'!F7:F66,"ano",'Hodnocení'!G7:G66,"&gt;=1",'Hodnocení'!G7:G66,"&lt;=5")</f>
-        <v/>
-      </c>
-      <c r="F19" s="15">
-        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G66,'Hodnocení'!B7:B66,A19,'Hodnocení'!D7:D66,C19,'Hodnocení'!F7:F66,"ano",'Hodnocení'!G7:G66,"&gt;=1",'Hodnocení'!G7:G66,"&lt;=5"),"")</f>
+      <c r="D20">
+        <f>COUNTIFS('Hodnocení'!B7:B71,A20,'Hodnocení'!D7:D71,C20,'Hodnocení'!F7:F71,"ano")</f>
+        <v/>
+      </c>
+      <c r="E20">
+        <f>COUNTIFS('Hodnocení'!B7:B71,A20,'Hodnocení'!D7:D71,C20,'Hodnocení'!F7:F71,"ano",'Hodnocení'!G7:G71,"&gt;=1",'Hodnocení'!G7:G71,"&lt;=5")</f>
+        <v/>
+      </c>
+      <c r="F20" s="15">
+        <f>IFERROR(AVERAGEIFS('Hodnocení'!G7:G71,'Hodnocení'!B7:B71,A20,'Hodnocení'!D7:D71,C20,'Hodnocení'!F7:F71,"ano",'Hodnocení'!G7:G71,"&gt;=1",'Hodnocení'!G7:G71,"&lt;=5"),"")</f>
         <v/>
       </c>
     </row>

</xml_diff>